<commit_message>
3 DEC 2025 CLOSING 2
</commit_message>
<xml_diff>
--- a/DECEMBER/DECEMBER FLOOR.xlsx
+++ b/DECEMBER/DECEMBER FLOOR.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19635" windowHeight="7500"/>
+    <workbookView windowWidth="19635" windowHeight="7500" firstSheet="1" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Anugrah (Bag, Cup, Box)" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="32">
   <si>
     <t>DATE</t>
   </si>
@@ -129,6 +129,12 @@
   </si>
   <si>
     <t>QTY</t>
+  </si>
+  <si>
+    <t>DISHY VANILA 5L</t>
+  </si>
+  <si>
+    <t>FLOOR CLEANER</t>
   </si>
   <si>
     <t>NO</t>
@@ -659,6 +665,19 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color auto="1"/>
@@ -679,17 +698,19 @@
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right/>
-      <top style="thin">
+      <right style="thin">
         <color auto="1"/>
-      </top>
+      </right>
+      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -719,28 +740,6 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
       <right style="thin">
         <color auto="1"/>
       </right>
@@ -752,13 +751,20 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="thin">
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
+      </left>
+      <right/>
+      <top style="thin">
         <color auto="1"/>
-      </bottom>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1040,7 +1046,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="129">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1081,16 +1087,16 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="178" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1102,39 +1108,45 @@
     <xf numFmtId="178" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="179" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="179" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="178" fontId="3" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="3" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="3" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="3" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="178" fontId="2" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="178" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1162,58 +1174,58 @@
     <xf numFmtId="181" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="181" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="181" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1226,7 +1238,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="180" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="178" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1235,30 +1247,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="182" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="0" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1272,7 +1284,7 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="178" fontId="8" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1281,7 +1293,7 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1306,7 +1318,7 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="181" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1318,40 +1330,40 @@
     <xf numFmtId="178" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="181" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="181" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="9" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="9" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="9" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="9" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="9" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="9" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1369,13 +1381,13 @@
     <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="9" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="9" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="178" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1387,7 +1399,7 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="178" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1574,6 +1586,50 @@
         <a:xfrm rot="16200000">
           <a:off x="6837045" y="6205220"/>
           <a:ext cx="3082925" cy="3879215"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>26035</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>56515</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>4355465</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>949325</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="ID_7BEFDB63F16448A5BB21710E631EB358" descr="WhatsApp Image 2025-12-03 at 11.37.37_bfde9d0a"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:srcRect l="6138" t="14811" b="10638"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="5956935" y="-131445"/>
+          <a:ext cx="3064510" cy="4329430"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1846,174 +1902,174 @@
   <dimension ref="A1:H9"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="18.75" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="17.4285714285714" style="89"/>
-    <col min="2" max="2" width="13.4285714285714" style="89" customWidth="1"/>
-    <col min="3" max="3" width="36" style="89" customWidth="1"/>
-    <col min="4" max="4" width="21.2857142857143" style="88" customWidth="1"/>
-    <col min="5" max="5" width="33.2857142857143" style="89" customWidth="1"/>
-    <col min="6" max="6" width="17.2857142857143" style="89" customWidth="1"/>
-    <col min="7" max="8" width="20.8571428571429" style="89" customWidth="1"/>
-    <col min="9" max="9" width="12.8571428571429" style="89"/>
-    <col min="10" max="10" width="12" style="89"/>
-    <col min="11" max="16384" width="18.0380952380952" style="89"/>
+    <col min="1" max="1" width="17.4285714285714" style="91"/>
+    <col min="2" max="2" width="13.4285714285714" style="91" customWidth="1"/>
+    <col min="3" max="3" width="36" style="91" customWidth="1"/>
+    <col min="4" max="4" width="21.2857142857143" style="90" customWidth="1"/>
+    <col min="5" max="5" width="33.2857142857143" style="91" customWidth="1"/>
+    <col min="6" max="6" width="17.2857142857143" style="91" customWidth="1"/>
+    <col min="7" max="8" width="20.8571428571429" style="91" customWidth="1"/>
+    <col min="9" max="9" width="12.8571428571429" style="91"/>
+    <col min="10" max="10" width="12" style="91"/>
+    <col min="11" max="16384" width="18.0380952380952" style="91"/>
   </cols>
   <sheetData>
-    <row r="1" s="87" customFormat="1" ht="16" customHeight="1" spans="1:8">
-      <c r="A1" s="114" t="s">
+    <row r="1" s="89" customFormat="1" ht="16" customHeight="1" spans="1:8">
+      <c r="A1" s="116" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="115" t="s">
+      <c r="B1" s="117" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="115" t="s">
+      <c r="C1" s="117" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="115" t="s">
+      <c r="D1" s="117" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="115" t="s">
+      <c r="E1" s="117" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="115" t="s">
+      <c r="F1" s="117" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="115" t="s">
+      <c r="G1" s="117" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="115" t="s">
+      <c r="H1" s="117" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" s="87" customFormat="1" ht="120" customHeight="1" spans="1:8">
-      <c r="A2" s="100">
+    <row r="2" s="89" customFormat="1" ht="120" customHeight="1" spans="1:8">
+      <c r="A2" s="102">
         <v>45994</v>
       </c>
-      <c r="B2" s="93">
+      <c r="B2" s="95">
         <v>2518</v>
       </c>
-      <c r="C2" s="116" t="s">
+      <c r="C2" s="118" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="117">
+      <c r="D2" s="119">
         <v>4</v>
       </c>
-      <c r="E2" s="95" t="str">
+      <c r="E2" s="97" t="str">
         <f>_xlfn.DISPIMG("ID_AF642E9448564DC2B9A94250BEBF50D7",1)</f>
         <v>=DISPIMG("ID_AF642E9448564DC2B9A94250BEBF50D7",1)</v>
       </c>
-      <c r="F2" s="96">
+      <c r="F2" s="98">
         <v>178000</v>
       </c>
-      <c r="G2" s="99">
-        <f>SUM(D2*F2)</f>
+      <c r="G2" s="101">
+        <f t="shared" ref="G2:G8" si="0">SUM(D2*F2)</f>
         <v>712000</v>
       </c>
-      <c r="H2" s="99">
+      <c r="H2" s="101">
         <f>SUM(G2:G3)</f>
         <v>1897000</v>
       </c>
     </row>
-    <row r="3" s="87" customFormat="1" ht="120" customHeight="1" spans="1:8">
-      <c r="A3" s="102"/>
-      <c r="B3" s="93"/>
-      <c r="C3" s="116" t="s">
+    <row r="3" s="89" customFormat="1" ht="120" customHeight="1" spans="1:8">
+      <c r="A3" s="104"/>
+      <c r="B3" s="95"/>
+      <c r="C3" s="118" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="117">
+      <c r="D3" s="119">
         <v>3</v>
       </c>
-      <c r="E3" s="105"/>
-      <c r="F3" s="96">
+      <c r="E3" s="107"/>
+      <c r="F3" s="98">
         <v>395000</v>
       </c>
-      <c r="G3" s="99">
-        <f>SUM(D3*F3)</f>
+      <c r="G3" s="101">
+        <f t="shared" si="0"/>
         <v>1185000</v>
       </c>
-      <c r="H3" s="106"/>
-    </row>
-    <row r="4" s="87" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A4" s="100"/>
-      <c r="B4" s="101"/>
-      <c r="C4" s="98"/>
-      <c r="D4" s="117"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="99"/>
-      <c r="G4" s="99">
-        <f>SUM(D4*F4)</f>
+      <c r="H3" s="108"/>
+    </row>
+    <row r="4" s="89" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A4" s="102"/>
+      <c r="B4" s="103"/>
+      <c r="C4" s="100"/>
+      <c r="D4" s="119"/>
+      <c r="E4" s="97"/>
+      <c r="F4" s="101"/>
+      <c r="G4" s="101">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H4" s="99">
+      <c r="H4" s="101">
         <f>SUM(G4:G7)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" s="87" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A5" s="102"/>
-      <c r="B5" s="103"/>
-      <c r="C5" s="93"/>
-      <c r="D5" s="93"/>
-      <c r="E5" s="105"/>
-      <c r="F5" s="118"/>
-      <c r="G5" s="99">
-        <f>SUM(D5*F5)</f>
+    <row r="5" s="89" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A5" s="104"/>
+      <c r="B5" s="105"/>
+      <c r="C5" s="95"/>
+      <c r="D5" s="95"/>
+      <c r="E5" s="107"/>
+      <c r="F5" s="120"/>
+      <c r="G5" s="101">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H5" s="106"/>
-    </row>
-    <row r="6" s="87" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A6" s="102"/>
-      <c r="B6" s="103"/>
-      <c r="C6" s="93"/>
-      <c r="D6" s="93"/>
-      <c r="E6" s="105"/>
-      <c r="F6" s="118"/>
-      <c r="G6" s="99">
-        <f>SUM(D6*F6)</f>
+      <c r="H5" s="108"/>
+    </row>
+    <row r="6" s="89" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A6" s="104"/>
+      <c r="B6" s="105"/>
+      <c r="C6" s="95"/>
+      <c r="D6" s="95"/>
+      <c r="E6" s="107"/>
+      <c r="F6" s="120"/>
+      <c r="G6" s="101">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="106"/>
-    </row>
-    <row r="7" s="87" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A7" s="102"/>
-      <c r="B7" s="103"/>
-      <c r="C7" s="101"/>
-      <c r="D7" s="101"/>
-      <c r="E7" s="105"/>
-      <c r="F7" s="118"/>
-      <c r="G7" s="99">
-        <f>SUM(D7*F7)</f>
+      <c r="H6" s="108"/>
+    </row>
+    <row r="7" s="89" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A7" s="104"/>
+      <c r="B7" s="105"/>
+      <c r="C7" s="103"/>
+      <c r="D7" s="103"/>
+      <c r="E7" s="107"/>
+      <c r="F7" s="120"/>
+      <c r="G7" s="101">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H7" s="106"/>
-    </row>
-    <row r="8" s="87" customFormat="1" ht="258" customHeight="1" spans="1:8">
-      <c r="A8" s="92"/>
-      <c r="B8" s="93"/>
-      <c r="C8" s="93"/>
-      <c r="D8" s="93"/>
-      <c r="E8" s="111"/>
-      <c r="F8" s="119"/>
-      <c r="G8" s="96">
-        <f>SUM(D8*F8)</f>
+      <c r="H7" s="108"/>
+    </row>
+    <row r="8" s="89" customFormat="1" ht="258" customHeight="1" spans="1:8">
+      <c r="A8" s="94"/>
+      <c r="B8" s="95"/>
+      <c r="C8" s="95"/>
+      <c r="D8" s="95"/>
+      <c r="E8" s="113"/>
+      <c r="F8" s="121"/>
+      <c r="G8" s="98">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="96">
+      <c r="H8" s="98">
         <f>SUM(G8)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9" s="87" customFormat="1" ht="18" customHeight="1" spans="1:8">
-      <c r="A9" s="120" t="s">
+    <row r="9" s="89" customFormat="1" ht="18" customHeight="1" spans="1:8">
+      <c r="A9" s="122" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="121"/>
-      <c r="C9" s="122"/>
-      <c r="D9" s="123"/>
-      <c r="E9" s="124"/>
-      <c r="F9" s="124"/>
-      <c r="G9" s="125"/>
-      <c r="H9" s="126">
+      <c r="B9" s="123"/>
+      <c r="C9" s="124"/>
+      <c r="D9" s="125"/>
+      <c r="E9" s="126"/>
+      <c r="F9" s="126"/>
+      <c r="G9" s="127"/>
+      <c r="H9" s="128">
         <f>SUM(H2:H8)</f>
         <v>1897000</v>
       </c>
@@ -2041,178 +2097,178 @@
   <dimension ref="A1:H8"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="18.75" outlineLevelRow="7" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="19.8571428571429" style="88"/>
-    <col min="2" max="2" width="18.8571428571429" style="88" customWidth="1"/>
-    <col min="3" max="3" width="43.0380952380952" style="88" customWidth="1"/>
-    <col min="4" max="4" width="14.4285714285714" style="88" customWidth="1"/>
-    <col min="5" max="5" width="58.9619047619048" style="89" customWidth="1"/>
-    <col min="6" max="6" width="19.5238095238095" style="89" customWidth="1"/>
-    <col min="7" max="8" width="20.8571428571429" style="89" customWidth="1"/>
-    <col min="9" max="9" width="12.8571428571429" style="89"/>
-    <col min="10" max="16384" width="9.14285714285714" style="89"/>
+    <col min="1" max="1" width="19.8571428571429" style="90"/>
+    <col min="2" max="2" width="18.8571428571429" style="90" customWidth="1"/>
+    <col min="3" max="3" width="43.0380952380952" style="90" customWidth="1"/>
+    <col min="4" max="4" width="14.4285714285714" style="90" customWidth="1"/>
+    <col min="5" max="5" width="58.9619047619048" style="91" customWidth="1"/>
+    <col min="6" max="6" width="19.5238095238095" style="91" customWidth="1"/>
+    <col min="7" max="8" width="20.8571428571429" style="91" customWidth="1"/>
+    <col min="9" max="9" width="12.8571428571429" style="91"/>
+    <col min="10" max="16384" width="9.14285714285714" style="91"/>
   </cols>
   <sheetData>
-    <row r="1" s="87" customFormat="1" ht="16" customHeight="1" spans="1:8">
-      <c r="A1" s="90" t="s">
+    <row r="1" s="89" customFormat="1" ht="16" customHeight="1" spans="1:8">
+      <c r="A1" s="92" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="91" t="s">
+      <c r="B1" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="91" t="s">
+      <c r="C1" s="93" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="91" t="s">
+      <c r="D1" s="93" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="91" t="s">
+      <c r="E1" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="91" t="s">
+      <c r="F1" s="93" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="91" t="s">
+      <c r="G1" s="93" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="91" t="s">
+      <c r="H1" s="93" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" s="87" customFormat="1" ht="249.35" customHeight="1" spans="1:8">
-      <c r="A2" s="92">
+    <row r="2" s="89" customFormat="1" ht="249.35" customHeight="1" spans="1:8">
+      <c r="A2" s="94">
         <v>45975</v>
       </c>
-      <c r="B2" s="93">
+      <c r="B2" s="95">
         <v>221</v>
       </c>
-      <c r="C2" s="94" t="s">
+      <c r="C2" s="96" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="94">
+      <c r="D2" s="96">
         <v>3</v>
       </c>
-      <c r="E2" s="95"/>
-      <c r="F2" s="96">
+      <c r="E2" s="97"/>
+      <c r="F2" s="98">
         <v>55000</v>
       </c>
-      <c r="G2" s="97">
+      <c r="G2" s="99">
         <f>D2*F2</f>
         <v>165000</v>
       </c>
-      <c r="H2" s="96">
+      <c r="H2" s="98">
         <f>SUM(G2:G2)</f>
         <v>165000</v>
       </c>
     </row>
-    <row r="3" s="87" customFormat="1" ht="251.35" customHeight="1" spans="1:8">
-      <c r="A3" s="92">
+    <row r="3" s="89" customFormat="1" ht="251.35" customHeight="1" spans="1:8">
+      <c r="A3" s="94">
         <v>45976</v>
       </c>
-      <c r="B3" s="93">
+      <c r="B3" s="95">
         <v>254</v>
       </c>
-      <c r="C3" s="98" t="s">
+      <c r="C3" s="100" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="94">
+      <c r="D3" s="96">
         <v>5</v>
       </c>
-      <c r="E3" s="95"/>
-      <c r="F3" s="97">
+      <c r="E3" s="97"/>
+      <c r="F3" s="99">
         <v>13000</v>
       </c>
-      <c r="G3" s="97">
+      <c r="G3" s="99">
         <f>D3*F3</f>
         <v>65000</v>
       </c>
-      <c r="H3" s="99">
+      <c r="H3" s="101">
         <f>SUM(G3:G3)</f>
         <v>65000</v>
       </c>
     </row>
-    <row r="4" s="87" customFormat="1" ht="83" customHeight="1" spans="1:8">
-      <c r="A4" s="100">
+    <row r="4" s="89" customFormat="1" ht="83" customHeight="1" spans="1:8">
+      <c r="A4" s="102">
         <v>45985</v>
       </c>
-      <c r="B4" s="101">
+      <c r="B4" s="103">
         <v>523</v>
       </c>
-      <c r="C4" s="98" t="s">
+      <c r="C4" s="100" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="94">
+      <c r="D4" s="96">
         <v>200</v>
       </c>
-      <c r="E4" s="95"/>
-      <c r="F4" s="97">
+      <c r="E4" s="97"/>
+      <c r="F4" s="99">
         <v>2300</v>
       </c>
-      <c r="G4" s="97">
+      <c r="G4" s="99">
         <f>D4*F4</f>
         <v>460000</v>
       </c>
-      <c r="H4" s="99">
+      <c r="H4" s="101">
         <f>SUM(G4:G6)</f>
         <v>1335000</v>
       </c>
     </row>
-    <row r="5" s="87" customFormat="1" ht="83" customHeight="1" spans="1:8">
-      <c r="A5" s="102"/>
-      <c r="B5" s="103"/>
-      <c r="C5" s="98" t="s">
+    <row r="5" s="89" customFormat="1" ht="83" customHeight="1" spans="1:8">
+      <c r="A5" s="104"/>
+      <c r="B5" s="105"/>
+      <c r="C5" s="100" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="104">
+      <c r="D5" s="106">
         <v>250</v>
       </c>
-      <c r="E5" s="105"/>
-      <c r="F5" s="99">
+      <c r="E5" s="107"/>
+      <c r="F5" s="101">
         <v>2000</v>
       </c>
-      <c r="G5" s="97">
+      <c r="G5" s="99">
         <f>D5*F5</f>
         <v>500000</v>
       </c>
-      <c r="H5" s="106"/>
-    </row>
-    <row r="6" s="87" customFormat="1" ht="83" customHeight="1" spans="1:8">
-      <c r="A6" s="107"/>
-      <c r="B6" s="108"/>
-      <c r="C6" s="98" t="s">
+      <c r="H5" s="108"/>
+    </row>
+    <row r="6" s="89" customFormat="1" ht="83" customHeight="1" spans="1:8">
+      <c r="A6" s="109"/>
+      <c r="B6" s="110"/>
+      <c r="C6" s="100" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="104">
+      <c r="D6" s="106">
         <v>150</v>
       </c>
-      <c r="E6" s="109"/>
-      <c r="F6" s="99">
+      <c r="E6" s="111"/>
+      <c r="F6" s="101">
         <v>2500</v>
       </c>
-      <c r="G6" s="97">
+      <c r="G6" s="99">
         <f>D6*F6</f>
         <v>375000</v>
       </c>
-      <c r="H6" s="110"/>
-    </row>
-    <row r="7" s="87" customFormat="1" ht="200" customHeight="1" spans="1:8">
-      <c r="A7" s="92"/>
-      <c r="B7" s="93"/>
-      <c r="C7" s="98"/>
-      <c r="D7" s="104"/>
-      <c r="E7" s="111"/>
-      <c r="F7" s="99"/>
-      <c r="G7" s="99"/>
-      <c r="H7" s="96"/>
-    </row>
-    <row r="8" s="87" customFormat="1" spans="1:8">
-      <c r="A8" s="112"/>
-      <c r="B8" s="112"/>
-      <c r="C8" s="112"/>
-      <c r="D8" s="112"/>
-      <c r="E8" s="112"/>
-      <c r="F8" s="112"/>
-      <c r="G8" s="113"/>
-      <c r="H8" s="113">
+      <c r="H6" s="112"/>
+    </row>
+    <row r="7" s="89" customFormat="1" ht="200" customHeight="1" spans="1:8">
+      <c r="A7" s="94"/>
+      <c r="B7" s="95"/>
+      <c r="C7" s="100"/>
+      <c r="D7" s="106"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="101"/>
+      <c r="G7" s="101"/>
+      <c r="H7" s="98"/>
+    </row>
+    <row r="8" s="89" customFormat="1" spans="1:8">
+      <c r="A8" s="114"/>
+      <c r="B8" s="114"/>
+      <c r="C8" s="114"/>
+      <c r="D8" s="114"/>
+      <c r="E8" s="114"/>
+      <c r="F8" s="114"/>
+      <c r="G8" s="115"/>
+      <c r="H8" s="115">
         <f>SUM(H2:H7)</f>
         <v>1565000</v>
       </c>
@@ -2247,184 +2303,184 @@
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="B1" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="51" t="s">
+      <c r="C1" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="51" t="s">
+      <c r="D1" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="51" t="s">
+      <c r="E1" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="51" t="s">
+      <c r="F1" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="51" t="s">
+      <c r="G1" s="53" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A2" s="52"/>
-      <c r="B2" s="39"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="57">
+      <c r="A2" s="54"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="59">
         <f>SUM(D2*F2)</f>
         <v>0</v>
       </c>
     </row>
     <row r="3" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A3" s="52"/>
-      <c r="B3" s="39"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="57"/>
+      <c r="A3" s="54"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="59"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="52"/>
-      <c r="B4" s="61" t="s">
+      <c r="A4" s="54"/>
+      <c r="B4" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="61"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62">
+      <c r="C4" s="63"/>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="64">
         <f>SUM(G2:G3)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="52"/>
-      <c r="B5" s="61" t="s">
+      <c r="A5" s="54"/>
+      <c r="B5" s="63" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="61"/>
-      <c r="D5" s="62"/>
-      <c r="E5" s="62"/>
-      <c r="F5" s="62"/>
-      <c r="G5" s="62">
+      <c r="C5" s="63"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64">
         <f>G4*11%</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="52"/>
-      <c r="B6" s="61" t="s">
+      <c r="A6" s="54"/>
+      <c r="B6" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="61"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="62"/>
-      <c r="F6" s="62"/>
-      <c r="G6" s="63">
+      <c r="C6" s="63"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="64"/>
+      <c r="F6" s="64"/>
+      <c r="G6" s="65">
         <v>243</v>
       </c>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="52"/>
-      <c r="B7" s="61" t="s">
+      <c r="A7" s="54"/>
+      <c r="B7" s="63" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="61"/>
-      <c r="D7" s="62"/>
-      <c r="E7" s="64"/>
-      <c r="F7" s="64"/>
-      <c r="G7" s="64">
+      <c r="C7" s="63"/>
+      <c r="D7" s="64"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
+      <c r="G7" s="66">
         <v>269482</v>
       </c>
     </row>
     <row r="8" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A8" s="52"/>
-      <c r="B8" s="65"/>
-      <c r="C8" s="66"/>
-      <c r="D8" s="67"/>
-      <c r="E8" s="68"/>
-      <c r="F8" s="42"/>
-      <c r="G8" s="69"/>
+      <c r="A8" s="54"/>
+      <c r="B8" s="67"/>
+      <c r="C8" s="68"/>
+      <c r="D8" s="69"/>
+      <c r="E8" s="70"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="71"/>
     </row>
     <row r="9" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A9" s="52"/>
-      <c r="B9" s="70"/>
-      <c r="C9" s="66"/>
-      <c r="D9" s="67"/>
-      <c r="E9" s="71"/>
-      <c r="F9" s="42"/>
-      <c r="G9" s="69"/>
+      <c r="A9" s="54"/>
+      <c r="B9" s="72"/>
+      <c r="C9" s="68"/>
+      <c r="D9" s="69"/>
+      <c r="E9" s="73"/>
+      <c r="F9" s="44"/>
+      <c r="G9" s="71"/>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="72"/>
-      <c r="B10" s="61" t="s">
+      <c r="A10" s="74"/>
+      <c r="B10" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="61"/>
-      <c r="D10" s="62"/>
-      <c r="E10" s="73"/>
-      <c r="F10" s="62"/>
-      <c r="G10" s="62">
+      <c r="C10" s="63"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="75"/>
+      <c r="F10" s="64"/>
+      <c r="G10" s="64">
         <f>SUM(G8:G9)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="74"/>
-      <c r="B11" s="75" t="s">
+      <c r="A11" s="76"/>
+      <c r="B11" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="76"/>
-      <c r="D11" s="62"/>
-      <c r="E11" s="73"/>
-      <c r="F11" s="62"/>
-      <c r="G11" s="62"/>
+      <c r="C11" s="78"/>
+      <c r="D11" s="64"/>
+      <c r="E11" s="75"/>
+      <c r="F11" s="64"/>
+      <c r="G11" s="64"/>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="72"/>
-      <c r="B12" s="61" t="s">
+      <c r="A12" s="74"/>
+      <c r="B12" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="61"/>
-      <c r="D12" s="62"/>
-      <c r="E12" s="73"/>
-      <c r="F12" s="62"/>
-      <c r="G12" s="63"/>
+      <c r="C12" s="63"/>
+      <c r="D12" s="64"/>
+      <c r="E12" s="75"/>
+      <c r="F12" s="64"/>
+      <c r="G12" s="65"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="77"/>
-      <c r="B13" s="78" t="s">
+      <c r="A13" s="79"/>
+      <c r="B13" s="80" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="79"/>
-      <c r="D13" s="62"/>
-      <c r="E13" s="64"/>
-      <c r="F13" s="80"/>
-      <c r="G13" s="64">
+      <c r="C13" s="81"/>
+      <c r="D13" s="64"/>
+      <c r="E13" s="66"/>
+      <c r="F13" s="82"/>
+      <c r="G13" s="66">
         <f>SUM(G10:G12)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="81" t="s">
+      <c r="A14" s="83" t="s">
         <v>10</v>
       </c>
-      <c r="B14" s="82"/>
-      <c r="C14" s="82"/>
-      <c r="D14" s="83"/>
-      <c r="E14" s="84">
+      <c r="B14" s="84"/>
+      <c r="C14" s="84"/>
+      <c r="D14" s="85"/>
+      <c r="E14" s="86">
         <f>G7+G13</f>
         <v>269482</v>
       </c>
-      <c r="F14" s="85"/>
-      <c r="G14" s="86"/>
+      <c r="F14" s="87"/>
+      <c r="G14" s="88"/>
     </row>
   </sheetData>
   <mergeCells count="20">
@@ -2461,253 +2517,253 @@
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="10.5714285714286" style="12" customWidth="1"/>
-    <col min="2" max="2" width="12.6" style="36" customWidth="1"/>
+    <col min="2" max="2" width="12.6" style="38" customWidth="1"/>
     <col min="3" max="3" width="36.1238095238095" style="12" customWidth="1"/>
     <col min="4" max="4" width="18.8285714285714" style="12" customWidth="1"/>
     <col min="5" max="5" width="12.2857142857143" style="12" customWidth="1"/>
     <col min="6" max="16384" width="9.14285714285714" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" s="35" customFormat="1" ht="19" customHeight="1" spans="1:5">
-      <c r="A1" s="37" t="s">
+    <row r="1" s="37" customFormat="1" ht="19" customHeight="1" spans="1:5">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="38" t="s">
+      <c r="B1" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="37" t="s">
+      <c r="C1" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="37" t="s">
+      <c r="D1" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="37" t="s">
+      <c r="E1" s="39" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" s="12" customFormat="1" ht="263.65" customHeight="1" spans="1:5">
-      <c r="A2" s="39"/>
-      <c r="B2" s="40"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="41"/>
+      <c r="A2" s="41"/>
+      <c r="B2" s="42"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="43"/>
     </row>
     <row r="3" s="12" customFormat="1" ht="255.1" customHeight="1" spans="1:5">
-      <c r="A3" s="39"/>
-      <c r="B3" s="40"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="44"/>
+      <c r="A3" s="41"/>
+      <c r="B3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="46"/>
     </row>
     <row r="4" s="12" customFormat="1" ht="249.95" customHeight="1" spans="1:5">
-      <c r="A4" s="39"/>
-      <c r="B4" s="40"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="44"/>
+      <c r="A4" s="41"/>
+      <c r="B4" s="42"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="46"/>
     </row>
     <row r="5" s="12" customFormat="1" ht="256.25" customHeight="1" spans="1:5">
-      <c r="A5" s="39"/>
-      <c r="B5" s="40"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="44"/>
+      <c r="A5" s="41"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="43"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="46"/>
     </row>
     <row r="6" s="12" customFormat="1" ht="253.85" customHeight="1" spans="1:5">
-      <c r="A6" s="39"/>
-      <c r="B6" s="40"/>
-      <c r="C6" s="41"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="44"/>
+      <c r="A6" s="41"/>
+      <c r="B6" s="42"/>
+      <c r="C6" s="43"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="46"/>
     </row>
     <row r="7" s="12" customFormat="1" ht="254.65" customHeight="1" spans="1:5">
-      <c r="A7" s="39"/>
-      <c r="B7" s="40"/>
-      <c r="C7" s="41"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="44"/>
+      <c r="A7" s="41"/>
+      <c r="B7" s="42"/>
+      <c r="C7" s="43"/>
+      <c r="D7" s="45"/>
+      <c r="E7" s="46"/>
     </row>
     <row r="8" s="12" customFormat="1" ht="255.35" customHeight="1" spans="1:5">
-      <c r="A8" s="39"/>
-      <c r="B8" s="40"/>
-      <c r="C8" s="41"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="44"/>
+      <c r="A8" s="41"/>
+      <c r="B8" s="42"/>
+      <c r="C8" s="43"/>
+      <c r="D8" s="45"/>
+      <c r="E8" s="46"/>
     </row>
     <row r="9" s="12" customFormat="1" ht="266.95" customHeight="1" spans="1:5">
-      <c r="A9" s="39"/>
-      <c r="B9" s="40"/>
-      <c r="C9" s="41"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="44"/>
+      <c r="A9" s="41"/>
+      <c r="B9" s="42"/>
+      <c r="C9" s="43"/>
+      <c r="D9" s="45"/>
+      <c r="E9" s="46"/>
     </row>
     <row r="10" s="12" customFormat="1" ht="261.95" customHeight="1" spans="1:5">
-      <c r="A10" s="39"/>
-      <c r="B10" s="40"/>
-      <c r="C10" s="41"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="44"/>
+      <c r="A10" s="41"/>
+      <c r="B10" s="42"/>
+      <c r="C10" s="43"/>
+      <c r="D10" s="45"/>
+      <c r="E10" s="46"/>
     </row>
     <row r="11" s="12" customFormat="1" ht="261.9" customHeight="1" spans="1:5">
-      <c r="A11" s="39"/>
-      <c r="B11" s="40"/>
-      <c r="C11" s="41"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="44"/>
+      <c r="A11" s="41"/>
+      <c r="B11" s="42"/>
+      <c r="C11" s="43"/>
+      <c r="D11" s="45"/>
+      <c r="E11" s="46"/>
     </row>
     <row r="12" s="12" customFormat="1" ht="270.7" customHeight="1" spans="1:5">
-      <c r="A12" s="39"/>
-      <c r="B12" s="40"/>
-      <c r="C12" s="41"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="44"/>
+      <c r="A12" s="41"/>
+      <c r="B12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="45"/>
+      <c r="E12" s="46"/>
     </row>
     <row r="13" s="12" customFormat="1" ht="261.1" customHeight="1" spans="1:5">
-      <c r="A13" s="39"/>
-      <c r="B13" s="40"/>
-      <c r="C13" s="41"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="44"/>
+      <c r="A13" s="41"/>
+      <c r="B13" s="42"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="45"/>
+      <c r="E13" s="46"/>
     </row>
     <row r="14" s="12" customFormat="1" ht="257.15" customHeight="1" spans="1:5">
-      <c r="A14" s="39"/>
-      <c r="B14" s="40"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="43"/>
-      <c r="E14" s="44"/>
+      <c r="A14" s="41"/>
+      <c r="B14" s="42"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="46"/>
     </row>
     <row r="15" s="12" customFormat="1" ht="263.55" customHeight="1" spans="1:5">
-      <c r="A15" s="39"/>
-      <c r="B15" s="40"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="43"/>
-      <c r="E15" s="44"/>
+      <c r="A15" s="41"/>
+      <c r="B15" s="42"/>
+      <c r="C15" s="43"/>
+      <c r="D15" s="45"/>
+      <c r="E15" s="46"/>
     </row>
     <row r="16" s="12" customFormat="1" ht="270.35" customHeight="1" spans="1:5">
-      <c r="A16" s="39"/>
-      <c r="B16" s="40"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="43"/>
-      <c r="E16" s="44"/>
+      <c r="A16" s="41"/>
+      <c r="B16" s="42"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="45"/>
+      <c r="E16" s="46"/>
     </row>
     <row r="17" s="12" customFormat="1" ht="261.7" customHeight="1" spans="1:5">
-      <c r="A17" s="39"/>
-      <c r="B17" s="40"/>
-      <c r="C17" s="41"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="44"/>
+      <c r="A17" s="41"/>
+      <c r="B17" s="42"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="45"/>
+      <c r="E17" s="46"/>
     </row>
     <row r="18" s="12" customFormat="1" ht="260" customHeight="1" spans="1:5">
-      <c r="A18" s="39"/>
-      <c r="B18" s="40"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="44"/>
+      <c r="A18" s="41"/>
+      <c r="B18" s="42"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="45"/>
+      <c r="E18" s="46"/>
     </row>
     <row r="19" s="12" customFormat="1" ht="263.2" customHeight="1" spans="1:5">
-      <c r="A19" s="39"/>
-      <c r="B19" s="40"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="44"/>
+      <c r="A19" s="41"/>
+      <c r="B19" s="42"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="45"/>
+      <c r="E19" s="46"/>
     </row>
     <row r="20" s="12" customFormat="1" ht="289.95" customHeight="1" spans="1:5">
-      <c r="A20" s="39"/>
-      <c r="B20" s="40"/>
-      <c r="C20" s="41"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="44"/>
+      <c r="A20" s="41"/>
+      <c r="B20" s="42"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="45"/>
+      <c r="E20" s="46"/>
     </row>
     <row r="21" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A21" s="39"/>
-      <c r="B21" s="40"/>
-      <c r="C21" s="41"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="44"/>
+      <c r="A21" s="41"/>
+      <c r="B21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="45"/>
+      <c r="E21" s="46"/>
     </row>
     <row r="22" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A22" s="39"/>
-      <c r="B22" s="40"/>
-      <c r="C22" s="41"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="44"/>
+      <c r="A22" s="41"/>
+      <c r="B22" s="42"/>
+      <c r="C22" s="43"/>
+      <c r="D22" s="45"/>
+      <c r="E22" s="46"/>
     </row>
     <row r="23" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A23" s="39"/>
-      <c r="B23" s="40"/>
-      <c r="C23" s="41"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="44"/>
+      <c r="A23" s="41"/>
+      <c r="B23" s="42"/>
+      <c r="C23" s="43"/>
+      <c r="D23" s="45"/>
+      <c r="E23" s="46"/>
     </row>
     <row r="24" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A24" s="39"/>
-      <c r="B24" s="40"/>
-      <c r="C24" s="41"/>
-      <c r="D24" s="42"/>
-      <c r="E24" s="41"/>
+      <c r="A24" s="41"/>
+      <c r="B24" s="42"/>
+      <c r="C24" s="43"/>
+      <c r="D24" s="44"/>
+      <c r="E24" s="43"/>
     </row>
     <row r="25" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A25" s="39"/>
-      <c r="B25" s="40"/>
-      <c r="C25" s="41"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="41"/>
+      <c r="A25" s="41"/>
+      <c r="B25" s="42"/>
+      <c r="C25" s="43"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="43"/>
     </row>
     <row r="26" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A26" s="39"/>
-      <c r="B26" s="40"/>
-      <c r="C26" s="41"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="41"/>
+      <c r="A26" s="41"/>
+      <c r="B26" s="42"/>
+      <c r="C26" s="43"/>
+      <c r="D26" s="44"/>
+      <c r="E26" s="43"/>
     </row>
     <row r="27" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A27" s="39">
+      <c r="A27" s="41">
         <v>45960</v>
       </c>
-      <c r="B27" s="40"/>
-      <c r="C27" s="41"/>
-      <c r="D27" s="42"/>
-      <c r="E27" s="41"/>
+      <c r="B27" s="42"/>
+      <c r="C27" s="43"/>
+      <c r="D27" s="44"/>
+      <c r="E27" s="43"/>
     </row>
     <row r="28" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A28" s="39">
+      <c r="A28" s="41">
         <v>45961</v>
       </c>
-      <c r="B28" s="40"/>
-      <c r="C28" s="41"/>
-      <c r="D28" s="42"/>
-      <c r="E28" s="41"/>
+      <c r="B28" s="42"/>
+      <c r="C28" s="43"/>
+      <c r="D28" s="44"/>
+      <c r="E28" s="43"/>
     </row>
     <row r="29" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A29" s="39"/>
-      <c r="B29" s="40"/>
-      <c r="C29" s="41"/>
-      <c r="D29" s="42"/>
-      <c r="E29" s="41"/>
+      <c r="A29" s="41"/>
+      <c r="B29" s="42"/>
+      <c r="C29" s="43"/>
+      <c r="D29" s="44"/>
+      <c r="E29" s="43"/>
     </row>
     <row r="30" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A30" s="39"/>
-      <c r="B30" s="40"/>
-      <c r="C30" s="41"/>
-      <c r="D30" s="42"/>
-      <c r="E30" s="41"/>
+      <c r="A30" s="41"/>
+      <c r="B30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="44"/>
+      <c r="E30" s="43"/>
     </row>
     <row r="31" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A31" s="39"/>
-      <c r="B31" s="40"/>
-      <c r="C31" s="41"/>
-      <c r="D31" s="42"/>
-      <c r="E31" s="41"/>
+      <c r="A31" s="41"/>
+      <c r="B31" s="42"/>
+      <c r="C31" s="43"/>
+      <c r="D31" s="44"/>
+      <c r="E31" s="43"/>
     </row>
     <row r="32" s="12" customFormat="1" spans="1:5">
-      <c r="A32" s="45"/>
-      <c r="B32" s="46"/>
-      <c r="C32" s="47">
+      <c r="A32" s="47"/>
+      <c r="B32" s="48"/>
+      <c r="C32" s="49">
         <f>SUM(D2:D31)</f>
         <v>0</v>
       </c>
-      <c r="D32" s="48"/>
-      <c r="E32" s="49"/>
+      <c r="D32" s="50"/>
+      <c r="E32" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2756,79 +2812,106 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" s="12" customFormat="1" ht="240.3" customHeight="1" spans="1:7">
-      <c r="A2" s="16"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="18"/>
+    <row r="2" s="12" customFormat="1" ht="171" customHeight="1" spans="1:7">
+      <c r="A2" s="16">
+        <v>45992</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="18">
+        <v>1</v>
+      </c>
       <c r="D2" s="19"/>
-      <c r="E2" s="20"/>
+      <c r="E2" s="20">
+        <v>60000</v>
+      </c>
       <c r="F2" s="21">
         <f>C2*E2</f>
-        <v>0</v>
+        <v>60000</v>
       </c>
       <c r="G2" s="22">
-        <f>SUM(F2:F2)</f>
-        <v>0</v>
+        <f>SUM(F2:F3)</f>
+        <v>115000</v>
       </c>
     </row>
     <row r="3" s="12" customFormat="1" ht="80" customHeight="1" spans="1:7">
       <c r="A3" s="23"/>
-      <c r="B3" s="24"/>
-      <c r="C3" s="25"/>
+      <c r="B3" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="25">
+        <v>1</v>
+      </c>
       <c r="D3" s="26"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="29"/>
+      <c r="E3" s="27">
+        <v>55000</v>
+      </c>
+      <c r="F3" s="21">
+        <f>C3*E3</f>
+        <v>55000</v>
+      </c>
+      <c r="G3" s="22"/>
     </row>
     <row r="4" s="12" customFormat="1" ht="80" customHeight="1" spans="1:7">
-      <c r="A4" s="23"/>
+      <c r="A4" s="28"/>
       <c r="B4" s="24"/>
       <c r="C4" s="25"/>
-      <c r="D4" s="26"/>
+      <c r="D4" s="29"/>
       <c r="E4" s="27"/>
-      <c r="F4" s="28"/>
+      <c r="F4" s="21">
+        <f>C4*E4</f>
+        <v>0</v>
+      </c>
       <c r="G4" s="30"/>
     </row>
     <row r="5" s="12" customFormat="1" ht="80" customHeight="1" spans="1:7">
-      <c r="A5" s="23"/>
+      <c r="A5" s="28"/>
       <c r="B5" s="24"/>
       <c r="C5" s="25"/>
-      <c r="D5" s="26"/>
+      <c r="D5" s="29"/>
       <c r="E5" s="27"/>
-      <c r="F5" s="28"/>
+      <c r="F5" s="21">
+        <f>C5*E5</f>
+        <v>0</v>
+      </c>
       <c r="G5" s="31"/>
     </row>
     <row r="6" s="12" customFormat="1" ht="23.25" spans="1:7">
-      <c r="A6" s="23"/>
+      <c r="A6" s="32"/>
       <c r="B6" s="24"/>
       <c r="C6" s="25"/>
-      <c r="D6" s="26"/>
+      <c r="D6" s="33"/>
       <c r="E6" s="27"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="32"/>
+      <c r="F6" s="21">
+        <f>C6*E6</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="31"/>
     </row>
     <row r="7" s="12" customFormat="1" ht="39" customHeight="1" spans="1:7">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="33"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="33"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="34">
+      <c r="B7" s="34"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="35"/>
+      <c r="G7" s="36">
         <f>SUM(G2:G6)</f>
-        <v>0</v>
+        <v>115000</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="D3:D5"/>
-    <mergeCell ref="G3:G5"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="G2:G3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2845,13 +2928,13 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:3">
       <c r="A1" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -2859,7 +2942,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" s="8">
         <f>'Anugrah (Bag, Cup, Box)'!H9</f>
@@ -2871,7 +2954,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C3" s="8">
         <f>'UD Abdi Jaya (Bag, Cup, Box)'!H8</f>
@@ -2883,7 +2966,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C4" s="8">
         <f>'PT. SUPARMA JAYA TBK (Tissue)'!E14</f>
@@ -2895,7 +2978,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C5" s="9">
         <f>'Vickel Laundry'!C32</f>
@@ -2907,11 +2990,11 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C6" s="9">
         <f>'Dishy Soap'!G7</f>
-        <v>0</v>
+        <v>115000</v>
       </c>
     </row>
     <row r="7" spans="1:3">

</xml_diff>

<commit_message>
6 DEC 2025 CLOSING
</commit_message>
<xml_diff>
--- a/DECEMBER/DECEMBER FLOOR.xlsx
+++ b/DECEMBER/DECEMBER FLOOR.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19635" windowHeight="7500" firstSheet="1" activeTab="4"/>
+    <workbookView windowWidth="19635" windowHeight="7500" firstSheet="2" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Anugrah (Bag, Cup, Box)" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="28">
   <si>
     <t>DATE</t>
   </si>
@@ -99,18 +99,6 @@
   </si>
   <si>
     <t>HAND GLOVES (M)</t>
-  </si>
-  <si>
-    <t>P KILAT 2</t>
-  </si>
-  <si>
-    <t>PAPER BAG L CB08</t>
-  </si>
-  <si>
-    <t>PAPER BAG S CB07</t>
-  </si>
-  <si>
-    <t>BURGER BOX XL</t>
   </si>
   <si>
     <t>SALES PRICE</t>
@@ -1476,128 +1464,6 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>27305</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>27305</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>3903345</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>3143885</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="ID_77CE357CEE334F6D961BD6780F917C7B" descr="WhatsApp Image 2025-11-17 at 19.55.24_b4d82a76"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:srcRect l="2094" t="17062" b="13764"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm rot="16200000">
-          <a:off x="6819900" y="-149225"/>
-          <a:ext cx="3116580" cy="3876040"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>31750</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>26035</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>3898900</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>3160395</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="ID_53A5575CEC60468792705E317509501C" descr="WhatsApp Image 2025-11-17 at 19.55.38_dd252dd0"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:srcRect l="877" t="19263" b="10630"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm rot="16200000">
-          <a:off x="6811010" y="3029585"/>
-          <a:ext cx="3134360" cy="3867150"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>26035</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>41275</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>3905250</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>1016000</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="ID_0EC8FE7F2FDE486BA9DB2B935A916937" descr="WhatsApp Image 2025-11-25 at 10.50.39_ab457d84"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:srcRect l="1551" t="17216" b="12348"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm rot="16200000">
-          <a:off x="6837045" y="6205220"/>
-          <a:ext cx="3082925" cy="3879215"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2161,92 +2027,60 @@
       </c>
     </row>
     <row r="3" s="89" customFormat="1" ht="251.35" customHeight="1" spans="1:8">
-      <c r="A3" s="94">
-        <v>45976</v>
-      </c>
-      <c r="B3" s="95">
-        <v>254</v>
-      </c>
-      <c r="C3" s="100" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="96">
-        <v>5</v>
-      </c>
+      <c r="A3" s="94"/>
+      <c r="B3" s="95"/>
+      <c r="C3" s="100"/>
+      <c r="D3" s="96"/>
       <c r="E3" s="97"/>
-      <c r="F3" s="99">
-        <v>13000</v>
-      </c>
+      <c r="F3" s="99"/>
       <c r="G3" s="99">
         <f>D3*F3</f>
-        <v>65000</v>
+        <v>0</v>
       </c>
       <c r="H3" s="101">
         <f>SUM(G3:G3)</f>
-        <v>65000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" s="89" customFormat="1" ht="83" customHeight="1" spans="1:8">
-      <c r="A4" s="102">
-        <v>45985</v>
-      </c>
-      <c r="B4" s="103">
-        <v>523</v>
-      </c>
-      <c r="C4" s="100" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="96">
-        <v>200</v>
-      </c>
+      <c r="A4" s="102"/>
+      <c r="B4" s="103"/>
+      <c r="C4" s="100"/>
+      <c r="D4" s="96"/>
       <c r="E4" s="97"/>
-      <c r="F4" s="99">
-        <v>2300</v>
-      </c>
+      <c r="F4" s="99"/>
       <c r="G4" s="99">
         <f>D4*F4</f>
-        <v>460000</v>
+        <v>0</v>
       </c>
       <c r="H4" s="101">
         <f>SUM(G4:G6)</f>
-        <v>1335000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" s="89" customFormat="1" ht="83" customHeight="1" spans="1:8">
       <c r="A5" s="104"/>
       <c r="B5" s="105"/>
-      <c r="C5" s="100" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="106">
-        <v>250</v>
-      </c>
+      <c r="C5" s="100"/>
+      <c r="D5" s="106"/>
       <c r="E5" s="107"/>
-      <c r="F5" s="101">
-        <v>2000</v>
-      </c>
+      <c r="F5" s="101"/>
       <c r="G5" s="99">
         <f>D5*F5</f>
-        <v>500000</v>
+        <v>0</v>
       </c>
       <c r="H5" s="108"/>
     </row>
     <row r="6" s="89" customFormat="1" ht="83" customHeight="1" spans="1:8">
       <c r="A6" s="109"/>
       <c r="B6" s="110"/>
-      <c r="C6" s="100" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="106">
-        <v>150</v>
-      </c>
+      <c r="C6" s="100"/>
+      <c r="D6" s="106"/>
       <c r="E6" s="111"/>
-      <c r="F6" s="101">
-        <v>2500</v>
-      </c>
+      <c r="F6" s="101"/>
       <c r="G6" s="99">
         <f>D6*F6</f>
-        <v>375000</v>
+        <v>0</v>
       </c>
       <c r="H6" s="112"/>
     </row>
@@ -2270,7 +2104,7 @@
       <c r="G8" s="115"/>
       <c r="H8" s="115">
         <f>SUM(H2:H7)</f>
-        <v>1565000</v>
+        <v>165000</v>
       </c>
     </row>
   </sheetData>
@@ -2283,7 +2117,6 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2349,7 +2182,7 @@
     <row r="4" spans="1:7">
       <c r="A4" s="54"/>
       <c r="B4" s="63" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C4" s="63"/>
       <c r="D4" s="64"/>
@@ -2363,7 +2196,7 @@
     <row r="5" spans="1:7">
       <c r="A5" s="54"/>
       <c r="B5" s="63" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C5" s="63"/>
       <c r="D5" s="64"/>
@@ -2377,7 +2210,7 @@
     <row r="6" spans="1:7">
       <c r="A6" s="54"/>
       <c r="B6" s="63" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C6" s="63"/>
       <c r="D6" s="64"/>
@@ -2421,7 +2254,7 @@
     <row r="10" spans="1:7">
       <c r="A10" s="74"/>
       <c r="B10" s="63" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C10" s="63"/>
       <c r="D10" s="64"/>
@@ -2435,7 +2268,7 @@
     <row r="11" spans="1:7">
       <c r="A11" s="76"/>
       <c r="B11" s="77" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C11" s="78"/>
       <c r="D11" s="64"/>
@@ -2446,7 +2279,7 @@
     <row r="12" spans="1:7">
       <c r="A12" s="74"/>
       <c r="B12" s="63" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C12" s="63"/>
       <c r="D12" s="64"/>
@@ -2538,7 +2371,7 @@
         <v>7</v>
       </c>
       <c r="E1" s="39" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" s="12" customFormat="1" ht="263.65" customHeight="1" spans="1:5">
@@ -2794,10 +2627,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D1" s="15" t="s">
         <v>4</v>
@@ -2817,7 +2650,7 @@
         <v>45992</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C2" s="18">
         <v>1</v>
@@ -2838,7 +2671,7 @@
     <row r="3" s="12" customFormat="1" ht="80" customHeight="1" spans="1:7">
       <c r="A3" s="23"/>
       <c r="B3" s="24" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C3" s="25">
         <v>1</v>
@@ -2928,13 +2761,13 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:3">
       <c r="A1" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -2942,7 +2775,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C2" s="8">
         <f>'Anugrah (Bag, Cup, Box)'!H9</f>
@@ -2954,11 +2787,11 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C3" s="8">
         <f>'UD Abdi Jaya (Bag, Cup, Box)'!H8</f>
-        <v>1565000</v>
+        <v>165000</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2966,7 +2799,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C4" s="8">
         <f>'PT. SUPARMA JAYA TBK (Tissue)'!E14</f>
@@ -2978,7 +2811,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C5" s="9">
         <f>'Vickel Laundry'!C32</f>
@@ -2990,7 +2823,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C6" s="9">
         <f>'Dishy Soap'!G7</f>
@@ -3004,7 +2837,7 @@
       <c r="B7" s="7"/>
       <c r="C7" s="10">
         <f>SUM(C2:C5)</f>
-        <v>3731482</v>
+        <v>2331482</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
20 DECEMBER 2025 19.38
</commit_message>
<xml_diff>
--- a/DECEMBER/DECEMBER FLOOR.xlsx
+++ b/DECEMBER/DECEMBER FLOOR.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19635" windowHeight="7500" firstSheet="1" activeTab="4"/>
+    <workbookView windowHeight="17000" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Anugrah (Bag, Cup, Box)" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="44">
   <si>
     <t>DATE</t>
   </si>
@@ -126,6 +126,12 @@
   </si>
   <si>
     <t>CUP HOLDER DOUBLE</t>
+  </si>
+  <si>
+    <t>0608</t>
+  </si>
+  <si>
+    <t>TOOTHPICK COVER PLAIN</t>
   </si>
   <si>
     <t>SALES PRICE</t>
@@ -196,16 +202,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="10">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="179" formatCode="[$-409]d\-mmm\-yyyy;@"/>
-    <numFmt numFmtId="180" formatCode="dd\-mmm"/>
-    <numFmt numFmtId="181" formatCode="_ [$IDR]\ * #,##0_ ;_ [$IDR]\ * \-#,##0_ ;_ [$IDR]\ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="182" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="183" formatCode="_-&quot;Rp&quot;* #,##0.00_-;\-&quot;Rp&quot;* #,##0.00_-;_-&quot;Rp&quot;* &quot;-&quot;??.00_-;_-@_-"/>
+    <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="180" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="181" formatCode="[$-409]d\-mmm\-yyyy;@"/>
+    <numFmt numFmtId="182" formatCode="dd\-mmm"/>
+    <numFmt numFmtId="183" formatCode="_ [$IDR]\ * #,##0_ ;_ [$IDR]\ * \-#,##0_ ;_ [$IDR]\ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="184" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="185" formatCode="_-&quot;Rp&quot;* #,##0.00_-;\-&quot;Rp&quot;* #,##0.00_-;_-&quot;Rp&quot;* &quot;-&quot;??.00_-;_-@_-"/>
   </numFmts>
   <fonts count="33">
     <font>
@@ -671,7 +677,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -712,19 +718,6 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -785,7 +778,9 @@
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -925,16 +920,16 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -943,7 +938,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -955,34 +950,34 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1067,7 +1062,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="134">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1088,30 +1083,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="178" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="180" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="180" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1120,55 +1115,49 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="3" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="3" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="2" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1183,7 +1172,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1192,27 +1181,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="183" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1222,96 +1211,96 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="183" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="180" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="178" fontId="8" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="184" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="185" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="184" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="180" fontId="8" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1334,7 +1323,7 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1346,61 +1335,70 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="181" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="181" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="9" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="9" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="183" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="11" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1409,46 +1407,49 @@
     <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="9" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="9" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1543,7 +1544,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm rot="5400000">
-          <a:off x="6958965" y="-283845"/>
+          <a:off x="8364220" y="-283845"/>
           <a:ext cx="2839085" cy="3867785"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1582,8 +1583,47 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm rot="16200000">
-          <a:off x="6939915" y="2624455"/>
+          <a:off x="8345170" y="2624455"/>
           <a:ext cx="2880995" cy="3891280"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>30797</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>26987</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>4770437</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>4471352</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="ID_FDB04E1C200E40C2A01C8C6D07A45482" descr="PHOTO-2025-12-17-17-40-21"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:srcRect l="2346" t="14598" b="17958"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="7995920" y="5921375"/>
+          <a:ext cx="4444365" cy="4739640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1626,7 +1666,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm rot="16200000">
-          <a:off x="6642735" y="-131445"/>
+          <a:off x="7953375" y="-131445"/>
           <a:ext cx="3064510" cy="4329430"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1665,7 +1705,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm rot="16200000">
-          <a:off x="6664325" y="2966085"/>
+          <a:off x="7974965" y="2966085"/>
           <a:ext cx="3006725" cy="4329430"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1937,176 +1977,176 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="18.75" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="20.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="17.4285714285714" style="92"/>
-    <col min="2" max="2" width="13.4285714285714" style="92" customWidth="1"/>
-    <col min="3" max="3" width="36" style="92" customWidth="1"/>
-    <col min="4" max="4" width="21.2857142857143" style="90" customWidth="1"/>
-    <col min="5" max="5" width="33.2857142857143" style="92" customWidth="1"/>
-    <col min="6" max="6" width="17.2857142857143" style="92" customWidth="1"/>
-    <col min="7" max="8" width="20.8571428571429" style="92" customWidth="1"/>
-    <col min="9" max="9" width="12.8571428571429" style="92"/>
-    <col min="10" max="10" width="12" style="92"/>
-    <col min="11" max="16384" width="18.0380952380952" style="92"/>
+    <col min="1" max="1" width="17.4296875" style="90"/>
+    <col min="2" max="2" width="13.4296875" style="90" customWidth="1"/>
+    <col min="3" max="3" width="36" style="90" customWidth="1"/>
+    <col min="4" max="4" width="21.2890625" style="88" customWidth="1"/>
+    <col min="5" max="5" width="33.2890625" style="90" customWidth="1"/>
+    <col min="6" max="6" width="17.2890625" style="90" customWidth="1"/>
+    <col min="7" max="8" width="20.859375" style="90" customWidth="1"/>
+    <col min="9" max="9" width="12.859375" style="90"/>
+    <col min="10" max="10" width="12" style="90"/>
+    <col min="11" max="16384" width="18.0390625" style="90"/>
   </cols>
   <sheetData>
-    <row r="1" s="89" customFormat="1" ht="16" customHeight="1" spans="1:8">
-      <c r="A1" s="119" t="s">
+    <row r="1" s="87" customFormat="1" ht="16" customHeight="1" spans="1:8">
+      <c r="A1" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="120" t="s">
+      <c r="B1" s="121" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="120" t="s">
+      <c r="C1" s="121" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="120" t="s">
+      <c r="D1" s="121" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="120" t="s">
+      <c r="E1" s="121" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="120" t="s">
+      <c r="F1" s="121" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="120" t="s">
+      <c r="G1" s="121" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="120" t="s">
+      <c r="H1" s="121" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" s="89" customFormat="1" ht="120" customHeight="1" spans="1:8">
-      <c r="A2" s="103">
+    <row r="2" s="87" customFormat="1" ht="120" customHeight="1" spans="1:8">
+      <c r="A2" s="98">
         <v>45994</v>
       </c>
-      <c r="B2" s="97">
+      <c r="B2" s="95">
         <v>2518</v>
       </c>
-      <c r="C2" s="121" t="s">
+      <c r="C2" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="122">
+      <c r="D2" s="123">
         <v>4</v>
       </c>
-      <c r="E2" s="100" t="str">
+      <c r="E2" s="110" t="str">
         <f>_xlfn.DISPIMG("ID_AF642E9448564DC2B9A94250BEBF50D7",1)</f>
         <v>=DISPIMG("ID_AF642E9448564DC2B9A94250BEBF50D7",1)</v>
       </c>
-      <c r="F2" s="101">
+      <c r="F2" s="111">
         <v>178000</v>
       </c>
-      <c r="G2" s="106">
+      <c r="G2" s="113">
         <f t="shared" ref="G2:G8" si="0">SUM(D2*F2)</f>
         <v>712000</v>
       </c>
-      <c r="H2" s="106">
+      <c r="H2" s="113">
         <f>SUM(G2:G3)</f>
         <v>1897000</v>
       </c>
     </row>
-    <row r="3" s="89" customFormat="1" ht="120" customHeight="1" spans="1:8">
-      <c r="A3" s="107"/>
-      <c r="B3" s="97"/>
-      <c r="C3" s="121" t="s">
+    <row r="3" s="87" customFormat="1" ht="120" customHeight="1" spans="1:8">
+      <c r="A3" s="101"/>
+      <c r="B3" s="95"/>
+      <c r="C3" s="122" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="122">
+      <c r="D3" s="123">
         <v>3</v>
       </c>
-      <c r="E3" s="109"/>
-      <c r="F3" s="101">
+      <c r="E3" s="114"/>
+      <c r="F3" s="111">
         <v>395000</v>
       </c>
-      <c r="G3" s="106">
+      <c r="G3" s="113">
         <f t="shared" si="0"/>
         <v>1185000</v>
       </c>
-      <c r="H3" s="110"/>
-    </row>
-    <row r="4" s="89" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A4" s="103"/>
-      <c r="B4" s="104"/>
-      <c r="C4" s="123"/>
-      <c r="D4" s="122"/>
-      <c r="E4" s="100"/>
-      <c r="F4" s="106"/>
-      <c r="G4" s="106">
+      <c r="H3" s="115"/>
+    </row>
+    <row r="4" s="87" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A4" s="98"/>
+      <c r="B4" s="99"/>
+      <c r="C4" s="124"/>
+      <c r="D4" s="123"/>
+      <c r="E4" s="110"/>
+      <c r="F4" s="113"/>
+      <c r="G4" s="113">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H4" s="106">
+      <c r="H4" s="113">
         <f>SUM(G4:G7)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" s="89" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A5" s="107"/>
-      <c r="B5" s="108"/>
-      <c r="C5" s="97"/>
-      <c r="D5" s="97"/>
-      <c r="E5" s="109"/>
-      <c r="F5" s="124"/>
-      <c r="G5" s="106">
+    <row r="5" s="87" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A5" s="101"/>
+      <c r="B5" s="102"/>
+      <c r="C5" s="95"/>
+      <c r="D5" s="95"/>
+      <c r="E5" s="114"/>
+      <c r="F5" s="129"/>
+      <c r="G5" s="113">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H5" s="110"/>
-    </row>
-    <row r="6" s="89" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A6" s="107"/>
-      <c r="B6" s="108"/>
-      <c r="C6" s="97"/>
-      <c r="D6" s="97"/>
-      <c r="E6" s="109"/>
-      <c r="F6" s="124"/>
-      <c r="G6" s="106">
+      <c r="H5" s="115"/>
+    </row>
+    <row r="6" s="87" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A6" s="101"/>
+      <c r="B6" s="102"/>
+      <c r="C6" s="95"/>
+      <c r="D6" s="95"/>
+      <c r="E6" s="114"/>
+      <c r="F6" s="129"/>
+      <c r="G6" s="113">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="110"/>
-    </row>
-    <row r="7" s="89" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A7" s="107"/>
-      <c r="B7" s="108"/>
-      <c r="C7" s="104"/>
-      <c r="D7" s="104"/>
-      <c r="E7" s="109"/>
-      <c r="F7" s="124"/>
-      <c r="G7" s="106">
+      <c r="H6" s="115"/>
+    </row>
+    <row r="7" s="87" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A7" s="101"/>
+      <c r="B7" s="102"/>
+      <c r="C7" s="99"/>
+      <c r="D7" s="99"/>
+      <c r="E7" s="114"/>
+      <c r="F7" s="129"/>
+      <c r="G7" s="113">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H7" s="110"/>
-    </row>
-    <row r="8" s="89" customFormat="1" ht="258" customHeight="1" spans="1:8">
-      <c r="A8" s="96"/>
-      <c r="B8" s="97"/>
-      <c r="C8" s="97"/>
-      <c r="D8" s="97"/>
-      <c r="E8" s="125"/>
-      <c r="F8" s="126"/>
-      <c r="G8" s="101">
+      <c r="H7" s="115"/>
+    </row>
+    <row r="8" s="87" customFormat="1" ht="258" customHeight="1" spans="1:8">
+      <c r="A8" s="94"/>
+      <c r="B8" s="95"/>
+      <c r="C8" s="95"/>
+      <c r="D8" s="95"/>
+      <c r="E8" s="130"/>
+      <c r="F8" s="131"/>
+      <c r="G8" s="111">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="101">
+      <c r="H8" s="111">
         <f>SUM(G8)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9" s="89" customFormat="1" ht="18" customHeight="1" spans="1:8">
-      <c r="A9" s="127" t="s">
+    <row r="9" s="87" customFormat="1" ht="18" customHeight="1" spans="1:8">
+      <c r="A9" s="125" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="128"/>
-      <c r="C9" s="129"/>
-      <c r="D9" s="130"/>
-      <c r="E9" s="131"/>
-      <c r="F9" s="131"/>
-      <c r="G9" s="132"/>
-      <c r="H9" s="133">
+      <c r="B9" s="126"/>
+      <c r="C9" s="127"/>
+      <c r="D9" s="128"/>
+      <c r="E9" s="132"/>
+      <c r="F9" s="132"/>
+      <c r="G9" s="133"/>
+      <c r="H9" s="134">
         <f>SUM(H2:H8)</f>
         <v>1897000</v>
       </c>
@@ -2131,247 +2171,273 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="18.75" outlineLevelCol="7"/>
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="20.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="19.8571428571429" style="90"/>
-    <col min="2" max="2" width="18.8571428571429" style="90" customWidth="1"/>
-    <col min="3" max="3" width="43.0380952380952" style="91" customWidth="1"/>
-    <col min="4" max="4" width="14.4285714285714" style="90" customWidth="1"/>
-    <col min="5" max="5" width="58.9619047619048" style="92" customWidth="1"/>
-    <col min="6" max="6" width="19.5238095238095" style="92" customWidth="1"/>
-    <col min="7" max="8" width="20.8571428571429" style="92" customWidth="1"/>
-    <col min="9" max="9" width="12.8571428571429" style="92"/>
-    <col min="10" max="16384" width="9.14285714285714" style="92"/>
+    <col min="1" max="1" width="19.859375" style="88"/>
+    <col min="2" max="2" width="18.859375" style="88" customWidth="1"/>
+    <col min="3" max="3" width="43.0390625" style="89" customWidth="1"/>
+    <col min="4" max="4" width="14.4296875" style="88" customWidth="1"/>
+    <col min="5" max="5" width="58.9609375" style="90" customWidth="1"/>
+    <col min="6" max="6" width="19.5234375" style="90" customWidth="1"/>
+    <col min="7" max="8" width="20.859375" style="90" customWidth="1"/>
+    <col min="9" max="9" width="12.859375" style="90"/>
+    <col min="10" max="16384" width="9.140625" style="90"/>
   </cols>
   <sheetData>
-    <row r="1" s="89" customFormat="1" ht="16" customHeight="1" spans="1:8">
-      <c r="A1" s="93" t="s">
+    <row r="1" s="87" customFormat="1" ht="16" customHeight="1" spans="1:8">
+      <c r="A1" s="91" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="94" t="s">
+      <c r="B1" s="92" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="95" t="s">
+      <c r="C1" s="93" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="94" t="s">
+      <c r="D1" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="94" t="s">
+      <c r="E1" s="92" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="94" t="s">
+      <c r="F1" s="92" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="94" t="s">
+      <c r="G1" s="92" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="94" t="s">
+      <c r="H1" s="92" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" s="89" customFormat="1" ht="227.8" customHeight="1" spans="1:8">
-      <c r="A2" s="96">
+    <row r="2" s="87" customFormat="1" ht="227.8" customHeight="1" spans="1:8">
+      <c r="A2" s="94">
         <v>45975</v>
       </c>
-      <c r="B2" s="97">
+      <c r="B2" s="95">
         <v>221</v>
       </c>
-      <c r="C2" s="98" t="s">
+      <c r="C2" s="96" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="99">
+      <c r="D2" s="97">
         <v>3</v>
       </c>
-      <c r="E2" s="100"/>
-      <c r="F2" s="101">
+      <c r="E2" s="110"/>
+      <c r="F2" s="111">
         <v>55000</v>
       </c>
-      <c r="G2" s="102">
-        <f t="shared" ref="G2:G10" si="0">D2*F2</f>
+      <c r="G2" s="112">
+        <f t="shared" ref="G2:G11" si="0">D2*F2</f>
         <v>165000</v>
       </c>
-      <c r="H2" s="101">
+      <c r="H2" s="111">
         <f>SUM(G2:G2)</f>
         <v>165000</v>
       </c>
     </row>
-    <row r="3" s="89" customFormat="1" ht="29" customHeight="1" spans="1:8">
-      <c r="A3" s="103">
+    <row r="3" s="87" customFormat="1" ht="29" customHeight="1" spans="1:8">
+      <c r="A3" s="98">
         <v>46002</v>
       </c>
-      <c r="B3" s="134" t="s">
+      <c r="B3" s="135" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="105" t="s">
+      <c r="C3" s="100" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="99">
+      <c r="D3" s="97">
         <v>1</v>
       </c>
-      <c r="E3" s="100"/>
-      <c r="F3" s="102">
+      <c r="E3" s="110"/>
+      <c r="F3" s="112">
         <v>295000</v>
       </c>
-      <c r="G3" s="102">
+      <c r="G3" s="112">
         <f t="shared" si="0"/>
         <v>295000</v>
       </c>
-      <c r="H3" s="106">
+      <c r="H3" s="113">
         <f>SUM(G3:G10)</f>
-        <v>4032500</v>
-      </c>
-    </row>
-    <row r="4" s="89" customFormat="1" ht="29" customHeight="1" spans="1:8">
-      <c r="A4" s="107"/>
-      <c r="B4" s="108"/>
-      <c r="C4" s="105" t="s">
+        <v>5280000</v>
+      </c>
+    </row>
+    <row r="4" s="87" customFormat="1" ht="29" customHeight="1" spans="1:8">
+      <c r="A4" s="101"/>
+      <c r="B4" s="102"/>
+      <c r="C4" s="100" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="99">
+      <c r="D4" s="97">
         <v>4</v>
       </c>
-      <c r="E4" s="109"/>
-      <c r="F4" s="102">
+      <c r="E4" s="114"/>
+      <c r="F4" s="112">
         <v>150000</v>
       </c>
-      <c r="G4" s="102">
+      <c r="G4" s="112">
         <f t="shared" si="0"/>
         <v>600000</v>
       </c>
-      <c r="H4" s="110"/>
-    </row>
-    <row r="5" s="89" customFormat="1" ht="29" customHeight="1" spans="1:8">
-      <c r="A5" s="107"/>
-      <c r="B5" s="108"/>
-      <c r="C5" s="105" t="s">
+      <c r="H4" s="115"/>
+    </row>
+    <row r="5" s="87" customFormat="1" ht="29" customHeight="1" spans="1:8">
+      <c r="A5" s="101"/>
+      <c r="B5" s="102"/>
+      <c r="C5" s="100" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="99">
+      <c r="D5" s="97">
         <v>4</v>
       </c>
-      <c r="E5" s="109"/>
-      <c r="F5" s="102">
+      <c r="E5" s="114"/>
+      <c r="F5" s="112">
         <v>460000</v>
       </c>
-      <c r="G5" s="102">
+      <c r="G5" s="112">
         <f t="shared" si="0"/>
         <v>1840000</v>
       </c>
-      <c r="H5" s="110"/>
-    </row>
-    <row r="6" s="89" customFormat="1" ht="29" customHeight="1" spans="1:8">
-      <c r="A6" s="107"/>
-      <c r="B6" s="108"/>
-      <c r="C6" s="105" t="s">
+      <c r="H5" s="115"/>
+    </row>
+    <row r="6" s="87" customFormat="1" ht="29" customHeight="1" spans="1:8">
+      <c r="A6" s="101"/>
+      <c r="B6" s="102"/>
+      <c r="C6" s="100" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="99">
+      <c r="D6" s="97">
         <v>2</v>
       </c>
-      <c r="E6" s="109"/>
-      <c r="F6" s="102">
+      <c r="E6" s="114"/>
+      <c r="F6" s="112">
         <v>340000</v>
       </c>
-      <c r="G6" s="102">
+      <c r="G6" s="112">
         <f t="shared" si="0"/>
         <v>680000</v>
       </c>
-      <c r="H6" s="110"/>
-    </row>
-    <row r="7" s="89" customFormat="1" ht="29" customHeight="1" spans="1:8">
-      <c r="A7" s="107"/>
-      <c r="B7" s="108"/>
-      <c r="C7" s="105" t="s">
+      <c r="H6" s="115"/>
+    </row>
+    <row r="7" s="87" customFormat="1" ht="29" customHeight="1" spans="1:8">
+      <c r="A7" s="101"/>
+      <c r="B7" s="102"/>
+      <c r="C7" s="100" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="99">
+      <c r="D7" s="97">
         <v>1</v>
       </c>
-      <c r="E7" s="109"/>
-      <c r="F7" s="101">
+      <c r="E7" s="114"/>
+      <c r="F7" s="111">
         <v>340000</v>
       </c>
-      <c r="G7" s="102">
+      <c r="G7" s="112">
         <f t="shared" si="0"/>
         <v>340000</v>
       </c>
-      <c r="H7" s="110"/>
-    </row>
-    <row r="8" s="89" customFormat="1" ht="29" customHeight="1" spans="1:8">
-      <c r="A8" s="107"/>
-      <c r="B8" s="108"/>
-      <c r="C8" s="111" t="s">
+      <c r="H7" s="115"/>
+    </row>
+    <row r="8" s="87" customFormat="1" ht="29" customHeight="1" spans="1:8">
+      <c r="A8" s="101"/>
+      <c r="B8" s="102"/>
+      <c r="C8" s="103" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="97">
+      <c r="D8" s="95">
         <v>5</v>
       </c>
-      <c r="E8" s="109"/>
-      <c r="F8" s="97">
+      <c r="E8" s="114"/>
+      <c r="F8" s="95">
         <v>55000</v>
       </c>
-      <c r="G8" s="102">
+      <c r="G8" s="112">
         <f t="shared" si="0"/>
         <v>275000</v>
       </c>
-      <c r="H8" s="110"/>
-    </row>
-    <row r="9" s="89" customFormat="1" ht="29" customHeight="1" spans="1:8">
-      <c r="A9" s="107"/>
-      <c r="B9" s="108"/>
-      <c r="C9" s="111" t="s">
+      <c r="H8" s="115"/>
+    </row>
+    <row r="9" s="87" customFormat="1" ht="29" customHeight="1" spans="1:8">
+      <c r="A9" s="101"/>
+      <c r="B9" s="102"/>
+      <c r="C9" s="103" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="97">
-        <v>1</v>
-      </c>
-      <c r="E9" s="109"/>
-      <c r="F9" s="97">
+      <c r="D9" s="95">
+        <v>500</v>
+      </c>
+      <c r="E9" s="114"/>
+      <c r="F9" s="95">
         <v>1000</v>
       </c>
-      <c r="G9" s="102">
+      <c r="G9" s="112">
         <f t="shared" si="0"/>
-        <v>1000</v>
-      </c>
-      <c r="H9" s="110"/>
-    </row>
-    <row r="10" s="89" customFormat="1" ht="29" customHeight="1" spans="1:8">
-      <c r="A10" s="112"/>
-      <c r="B10" s="113"/>
-      <c r="C10" s="111" t="s">
+        <v>500000</v>
+      </c>
+      <c r="H9" s="115"/>
+    </row>
+    <row r="10" s="87" customFormat="1" ht="29" customHeight="1" spans="1:8">
+      <c r="A10" s="104"/>
+      <c r="B10" s="105"/>
+      <c r="C10" s="103" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="97">
-        <v>1</v>
-      </c>
-      <c r="E10" s="114"/>
-      <c r="F10" s="97">
+      <c r="D10" s="95">
+        <v>500</v>
+      </c>
+      <c r="E10" s="116"/>
+      <c r="F10" s="95">
         <v>1500</v>
       </c>
-      <c r="G10" s="102">
+      <c r="G10" s="112">
         <f t="shared" si="0"/>
-        <v>1500</v>
-      </c>
-      <c r="H10" s="115"/>
-    </row>
-    <row r="11" s="89" customFormat="1" spans="1:8">
-      <c r="A11" s="116"/>
-      <c r="B11" s="116"/>
-      <c r="C11" s="117"/>
-      <c r="D11" s="116"/>
-      <c r="E11" s="116"/>
-      <c r="F11" s="116"/>
-      <c r="G11" s="118"/>
+        <v>750000</v>
+      </c>
+      <c r="H10" s="117"/>
+    </row>
+    <row r="11" s="87" customFormat="1" ht="353.9" customHeight="1" spans="1:8">
+      <c r="A11" s="106">
+        <v>46008</v>
+      </c>
+      <c r="B11" s="136" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="108" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="109">
+        <v>20</v>
+      </c>
+      <c r="E11" s="107"/>
+      <c r="F11" s="109">
+        <v>25000</v>
+      </c>
+      <c r="G11" s="112">
+        <f t="shared" si="0"/>
+        <v>500000</v>
+      </c>
       <c r="H11" s="118">
-        <f>SUM(H2:H10)</f>
-        <v>4197500</v>
+        <f>SUM(G11)</f>
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="12" s="87" customFormat="1" spans="1:8">
+      <c r="A12" s="109"/>
+      <c r="B12" s="109"/>
+      <c r="C12" s="108"/>
+      <c r="D12" s="109"/>
+      <c r="E12" s="109"/>
+      <c r="F12" s="109"/>
+      <c r="G12" s="112"/>
+      <c r="H12" s="119">
+        <f>SUM(H2:H11)</f>
+        <v>5945000</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A12:E12"/>
     <mergeCell ref="A3:A10"/>
     <mergeCell ref="B3:B10"/>
     <mergeCell ref="E3:E10"/>
@@ -2387,194 +2453,194 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="11.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="22.1428571428571" customWidth="1"/>
-    <col min="3" max="3" width="22.5714285714286" customWidth="1"/>
-    <col min="4" max="4" width="17.5714285714286" customWidth="1"/>
-    <col min="5" max="5" width="34.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="19.4285714285714" customWidth="1"/>
-    <col min="7" max="7" width="17.2857142857143" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="2" max="2" width="22.140625" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" customWidth="1"/>
+    <col min="5" max="5" width="34.5703125" customWidth="1"/>
+    <col min="6" max="6" width="19.4296875" customWidth="1"/>
+    <col min="7" max="7" width="17.2890625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="53" t="s">
+      <c r="B1" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="53" t="s">
+      <c r="C1" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="53" t="s">
+      <c r="D1" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="53" t="s">
+      <c r="E1" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="53" t="s">
+      <c r="F1" s="51" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="53" t="s">
+      <c r="G1" s="51" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A2" s="54"/>
-      <c r="B2" s="41"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="59">
+      <c r="A2" s="52"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="74"/>
+      <c r="G2" s="75">
         <f>SUM(D2*F2)</f>
         <v>0</v>
       </c>
     </row>
     <row r="3" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A3" s="54"/>
-      <c r="B3" s="41"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="59"/>
+      <c r="A3" s="52"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="73"/>
+      <c r="F3" s="76"/>
+      <c r="G3" s="75"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="54"/>
-      <c r="B4" s="63" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="63"/>
-      <c r="D4" s="64"/>
-      <c r="E4" s="64"/>
-      <c r="F4" s="64"/>
-      <c r="G4" s="64">
+      <c r="A4" s="52"/>
+      <c r="B4" s="57" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="57"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58">
         <f>SUM(G2:G3)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="54"/>
-      <c r="B5" s="63" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="63"/>
-      <c r="D5" s="64"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
-      <c r="G5" s="64">
+      <c r="A5" s="52"/>
+      <c r="B5" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="57"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="58"/>
+      <c r="F5" s="58"/>
+      <c r="G5" s="58">
         <f>G4*11%</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="54"/>
-      <c r="B6" s="63" t="s">
+      <c r="A6" s="52"/>
+      <c r="B6" s="57" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="57"/>
+      <c r="D6" s="58"/>
+      <c r="E6" s="58"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="77">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="52"/>
+      <c r="B7" s="57" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="57"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="78"/>
+      <c r="F7" s="78"/>
+      <c r="G7" s="78"/>
+    </row>
+    <row r="8" ht="123.5" customHeight="1" spans="1:7">
+      <c r="A8" s="52"/>
+      <c r="B8" s="59"/>
+      <c r="C8" s="60"/>
+      <c r="D8" s="61"/>
+      <c r="E8" s="79"/>
+      <c r="F8" s="42"/>
+      <c r="G8" s="80"/>
+    </row>
+    <row r="9" ht="123.5" customHeight="1" spans="1:7">
+      <c r="A9" s="52"/>
+      <c r="B9" s="62"/>
+      <c r="C9" s="60"/>
+      <c r="D9" s="61"/>
+      <c r="E9" s="81"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="80"/>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="63"/>
+      <c r="B10" s="57" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="63"/>
-      <c r="D6" s="64"/>
-      <c r="E6" s="64"/>
-      <c r="F6" s="64"/>
-      <c r="G6" s="65">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="54"/>
-      <c r="B7" s="63" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="63"/>
-      <c r="D7" s="64"/>
-      <c r="E7" s="66"/>
-      <c r="F7" s="66"/>
-      <c r="G7" s="66"/>
-    </row>
-    <row r="8" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A8" s="54"/>
-      <c r="B8" s="67"/>
-      <c r="C8" s="68"/>
-      <c r="D8" s="69"/>
-      <c r="E8" s="70"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="71"/>
-    </row>
-    <row r="9" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A9" s="54"/>
-      <c r="B9" s="72"/>
-      <c r="C9" s="68"/>
-      <c r="D9" s="69"/>
-      <c r="E9" s="73"/>
-      <c r="F9" s="44"/>
-      <c r="G9" s="71"/>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="74"/>
-      <c r="B10" s="63" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="63"/>
-      <c r="D10" s="64"/>
-      <c r="E10" s="75"/>
-      <c r="F10" s="64"/>
-      <c r="G10" s="64">
+      <c r="C10" s="57"/>
+      <c r="D10" s="58"/>
+      <c r="E10" s="82"/>
+      <c r="F10" s="58"/>
+      <c r="G10" s="58">
         <f>SUM(G8:G9)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="76"/>
-      <c r="B11" s="77" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="78"/>
-      <c r="D11" s="64"/>
-      <c r="E11" s="75"/>
-      <c r="F11" s="64"/>
-      <c r="G11" s="64"/>
+      <c r="A11" s="64"/>
+      <c r="B11" s="65" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="66"/>
+      <c r="D11" s="58"/>
+      <c r="E11" s="82"/>
+      <c r="F11" s="58"/>
+      <c r="G11" s="58"/>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="74"/>
-      <c r="B12" s="63" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="63"/>
-      <c r="D12" s="64"/>
-      <c r="E12" s="75"/>
-      <c r="F12" s="64"/>
-      <c r="G12" s="65"/>
+      <c r="A12" s="63"/>
+      <c r="B12" s="57" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="57"/>
+      <c r="D12" s="58"/>
+      <c r="E12" s="82"/>
+      <c r="F12" s="58"/>
+      <c r="G12" s="77"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="79"/>
-      <c r="B13" s="80" t="s">
+      <c r="A13" s="67"/>
+      <c r="B13" s="68" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="81"/>
-      <c r="D13" s="64"/>
-      <c r="E13" s="66"/>
-      <c r="F13" s="82"/>
-      <c r="G13" s="66">
+      <c r="C13" s="69"/>
+      <c r="D13" s="58"/>
+      <c r="E13" s="78"/>
+      <c r="F13" s="83"/>
+      <c r="G13" s="78">
         <f>SUM(G10:G12)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="83" t="s">
+      <c r="A14" s="70" t="s">
         <v>10</v>
       </c>
-      <c r="B14" s="84"/>
-      <c r="C14" s="84"/>
-      <c r="D14" s="85"/>
-      <c r="E14" s="86">
+      <c r="B14" s="71"/>
+      <c r="C14" s="71"/>
+      <c r="D14" s="72"/>
+      <c r="E14" s="84">
         <f>G7+G13</f>
         <v>0</v>
       </c>
-      <c r="F14" s="87"/>
-      <c r="G14" s="88"/>
+      <c r="F14" s="85"/>
+      <c r="G14" s="86"/>
     </row>
   </sheetData>
   <mergeCells count="20">
@@ -2608,256 +2674,256 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E32"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="10.5714285714286" style="12" customWidth="1"/>
-    <col min="2" max="2" width="12.6" style="38" customWidth="1"/>
-    <col min="3" max="3" width="36.1238095238095" style="12" customWidth="1"/>
-    <col min="4" max="4" width="18.8285714285714" style="12" customWidth="1"/>
-    <col min="5" max="5" width="12.2857142857143" style="12" customWidth="1"/>
-    <col min="6" max="16384" width="9.14285714285714" style="12"/>
+    <col min="1" max="1" width="10.5703125" style="12" customWidth="1"/>
+    <col min="2" max="2" width="12.6015625" style="36" customWidth="1"/>
+    <col min="3" max="3" width="36.125" style="12" customWidth="1"/>
+    <col min="4" max="4" width="18.828125" style="12" customWidth="1"/>
+    <col min="5" max="5" width="12.2890625" style="12" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" s="37" customFormat="1" ht="19" customHeight="1" spans="1:5">
-      <c r="A1" s="39" t="s">
+    <row r="1" s="35" customFormat="1" ht="19" customHeight="1" spans="1:5">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="39" t="s">
+      <c r="C1" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="39" t="s">
+      <c r="D1" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="39" t="s">
-        <v>24</v>
+      <c r="E1" s="37" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="2" s="12" customFormat="1" ht="263.65" customHeight="1" spans="1:5">
-      <c r="A2" s="41"/>
-      <c r="B2" s="42"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="43"/>
+      <c r="A2" s="39"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="41"/>
     </row>
     <row r="3" s="12" customFormat="1" ht="255.1" customHeight="1" spans="1:5">
-      <c r="A3" s="41"/>
-      <c r="B3" s="42"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="46"/>
+      <c r="A3" s="39"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="48"/>
     </row>
     <row r="4" s="12" customFormat="1" ht="249.95" customHeight="1" spans="1:5">
-      <c r="A4" s="41"/>
-      <c r="B4" s="42"/>
-      <c r="C4" s="43"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="46"/>
+      <c r="A4" s="39"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="48"/>
     </row>
     <row r="5" s="12" customFormat="1" ht="256.25" customHeight="1" spans="1:5">
-      <c r="A5" s="41"/>
-      <c r="B5" s="42"/>
-      <c r="C5" s="43"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="46"/>
+      <c r="A5" s="39"/>
+      <c r="B5" s="40"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="48"/>
     </row>
     <row r="6" s="12" customFormat="1" ht="253.85" customHeight="1" spans="1:5">
-      <c r="A6" s="41"/>
-      <c r="B6" s="42"/>
-      <c r="C6" s="43"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="46"/>
+      <c r="A6" s="39"/>
+      <c r="B6" s="40"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="48"/>
     </row>
     <row r="7" s="12" customFormat="1" ht="254.65" customHeight="1" spans="1:5">
-      <c r="A7" s="41"/>
-      <c r="B7" s="42"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="46"/>
+      <c r="A7" s="39"/>
+      <c r="B7" s="40"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="48"/>
     </row>
     <row r="8" s="12" customFormat="1" ht="255.35" customHeight="1" spans="1:5">
-      <c r="A8" s="41"/>
-      <c r="B8" s="42"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="45"/>
-      <c r="E8" s="46"/>
+      <c r="A8" s="39"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="48"/>
     </row>
     <row r="9" s="12" customFormat="1" ht="266.95" customHeight="1" spans="1:5">
-      <c r="A9" s="41"/>
-      <c r="B9" s="42"/>
-      <c r="C9" s="43"/>
-      <c r="D9" s="45"/>
-      <c r="E9" s="46"/>
+      <c r="A9" s="39"/>
+      <c r="B9" s="40"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="48"/>
     </row>
     <row r="10" s="12" customFormat="1" ht="261.95" customHeight="1" spans="1:5">
-      <c r="A10" s="41"/>
-      <c r="B10" s="42"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="45"/>
-      <c r="E10" s="46"/>
+      <c r="A10" s="39"/>
+      <c r="B10" s="40"/>
+      <c r="C10" s="41"/>
+      <c r="D10" s="43"/>
+      <c r="E10" s="48"/>
     </row>
     <row r="11" s="12" customFormat="1" ht="261.9" customHeight="1" spans="1:5">
-      <c r="A11" s="41"/>
-      <c r="B11" s="42"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="46"/>
+      <c r="A11" s="39"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="48"/>
     </row>
     <row r="12" s="12" customFormat="1" ht="270.7" customHeight="1" spans="1:5">
-      <c r="A12" s="41"/>
-      <c r="B12" s="42"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="45"/>
-      <c r="E12" s="46"/>
+      <c r="A12" s="39"/>
+      <c r="B12" s="40"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="48"/>
     </row>
     <row r="13" s="12" customFormat="1" ht="261.1" customHeight="1" spans="1:5">
-      <c r="A13" s="41"/>
-      <c r="B13" s="42"/>
-      <c r="C13" s="43"/>
-      <c r="D13" s="45"/>
-      <c r="E13" s="46"/>
+      <c r="A13" s="39"/>
+      <c r="B13" s="40"/>
+      <c r="C13" s="41"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="48"/>
     </row>
     <row r="14" s="12" customFormat="1" ht="257.15" customHeight="1" spans="1:5">
-      <c r="A14" s="41"/>
-      <c r="B14" s="42"/>
-      <c r="C14" s="43"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="46"/>
+      <c r="A14" s="39"/>
+      <c r="B14" s="40"/>
+      <c r="C14" s="41"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="48"/>
     </row>
     <row r="15" s="12" customFormat="1" ht="263.55" customHeight="1" spans="1:5">
-      <c r="A15" s="41"/>
-      <c r="B15" s="42"/>
-      <c r="C15" s="43"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="46"/>
+      <c r="A15" s="39"/>
+      <c r="B15" s="40"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="43"/>
+      <c r="E15" s="48"/>
     </row>
     <row r="16" s="12" customFormat="1" ht="270.35" customHeight="1" spans="1:5">
-      <c r="A16" s="41"/>
-      <c r="B16" s="42"/>
-      <c r="C16" s="43"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="46"/>
+      <c r="A16" s="39"/>
+      <c r="B16" s="40"/>
+      <c r="C16" s="41"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="48"/>
     </row>
     <row r="17" s="12" customFormat="1" ht="261.7" customHeight="1" spans="1:5">
-      <c r="A17" s="41"/>
-      <c r="B17" s="42"/>
-      <c r="C17" s="43"/>
-      <c r="D17" s="45"/>
-      <c r="E17" s="46"/>
+      <c r="A17" s="39"/>
+      <c r="B17" s="40"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="48"/>
     </row>
     <row r="18" s="12" customFormat="1" ht="260" customHeight="1" spans="1:5">
-      <c r="A18" s="41"/>
-      <c r="B18" s="42"/>
-      <c r="C18" s="43"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="46"/>
+      <c r="A18" s="39"/>
+      <c r="B18" s="40"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="48"/>
     </row>
     <row r="19" s="12" customFormat="1" ht="263.2" customHeight="1" spans="1:5">
-      <c r="A19" s="41"/>
-      <c r="B19" s="42"/>
-      <c r="C19" s="43"/>
-      <c r="D19" s="45"/>
-      <c r="E19" s="46"/>
+      <c r="A19" s="39"/>
+      <c r="B19" s="40"/>
+      <c r="C19" s="41"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="48"/>
     </row>
     <row r="20" s="12" customFormat="1" ht="289.95" customHeight="1" spans="1:5">
-      <c r="A20" s="41"/>
-      <c r="B20" s="42"/>
-      <c r="C20" s="43"/>
-      <c r="D20" s="45"/>
-      <c r="E20" s="46"/>
+      <c r="A20" s="39"/>
+      <c r="B20" s="40"/>
+      <c r="C20" s="41"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="48"/>
     </row>
     <row r="21" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A21" s="41"/>
-      <c r="B21" s="42"/>
-      <c r="C21" s="43"/>
-      <c r="D21" s="45"/>
-      <c r="E21" s="46"/>
+      <c r="A21" s="39"/>
+      <c r="B21" s="40"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="48"/>
     </row>
     <row r="22" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A22" s="41"/>
-      <c r="B22" s="42"/>
-      <c r="C22" s="43"/>
-      <c r="D22" s="45"/>
-      <c r="E22" s="46"/>
+      <c r="A22" s="39"/>
+      <c r="B22" s="40"/>
+      <c r="C22" s="41"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="48"/>
     </row>
     <row r="23" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A23" s="41"/>
-      <c r="B23" s="42"/>
-      <c r="C23" s="43"/>
-      <c r="D23" s="45"/>
-      <c r="E23" s="46"/>
+      <c r="A23" s="39"/>
+      <c r="B23" s="40"/>
+      <c r="C23" s="41"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="48"/>
     </row>
     <row r="24" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A24" s="41"/>
-      <c r="B24" s="42"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="44"/>
-      <c r="E24" s="43"/>
+      <c r="A24" s="39"/>
+      <c r="B24" s="40"/>
+      <c r="C24" s="41"/>
+      <c r="D24" s="42"/>
+      <c r="E24" s="41"/>
     </row>
     <row r="25" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A25" s="41"/>
-      <c r="B25" s="42"/>
-      <c r="C25" s="43"/>
-      <c r="D25" s="44"/>
-      <c r="E25" s="43"/>
+      <c r="A25" s="39"/>
+      <c r="B25" s="40"/>
+      <c r="C25" s="41"/>
+      <c r="D25" s="42"/>
+      <c r="E25" s="41"/>
     </row>
     <row r="26" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A26" s="41"/>
-      <c r="B26" s="42"/>
-      <c r="C26" s="43"/>
-      <c r="D26" s="44"/>
-      <c r="E26" s="43"/>
+      <c r="A26" s="39"/>
+      <c r="B26" s="40"/>
+      <c r="C26" s="41"/>
+      <c r="D26" s="42"/>
+      <c r="E26" s="41"/>
     </row>
     <row r="27" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A27" s="41">
+      <c r="A27" s="39">
         <v>45960</v>
       </c>
-      <c r="B27" s="42"/>
-      <c r="C27" s="43"/>
-      <c r="D27" s="44"/>
-      <c r="E27" s="43"/>
+      <c r="B27" s="40"/>
+      <c r="C27" s="41"/>
+      <c r="D27" s="42"/>
+      <c r="E27" s="41"/>
     </row>
     <row r="28" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A28" s="41">
+      <c r="A28" s="39">
         <v>45961</v>
       </c>
-      <c r="B28" s="42"/>
-      <c r="C28" s="43"/>
-      <c r="D28" s="44"/>
-      <c r="E28" s="43"/>
+      <c r="B28" s="40"/>
+      <c r="C28" s="41"/>
+      <c r="D28" s="42"/>
+      <c r="E28" s="41"/>
     </row>
     <row r="29" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A29" s="41"/>
-      <c r="B29" s="42"/>
-      <c r="C29" s="43"/>
-      <c r="D29" s="44"/>
-      <c r="E29" s="43"/>
+      <c r="A29" s="39"/>
+      <c r="B29" s="40"/>
+      <c r="C29" s="41"/>
+      <c r="D29" s="42"/>
+      <c r="E29" s="41"/>
     </row>
     <row r="30" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A30" s="41"/>
-      <c r="B30" s="42"/>
-      <c r="C30" s="43"/>
-      <c r="D30" s="44"/>
-      <c r="E30" s="43"/>
+      <c r="A30" s="39"/>
+      <c r="B30" s="40"/>
+      <c r="C30" s="41"/>
+      <c r="D30" s="42"/>
+      <c r="E30" s="41"/>
     </row>
     <row r="31" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A31" s="41"/>
-      <c r="B31" s="42"/>
-      <c r="C31" s="43"/>
-      <c r="D31" s="44"/>
-      <c r="E31" s="43"/>
+      <c r="A31" s="39"/>
+      <c r="B31" s="40"/>
+      <c r="C31" s="41"/>
+      <c r="D31" s="42"/>
+      <c r="E31" s="41"/>
     </row>
     <row r="32" s="12" customFormat="1" spans="1:5">
-      <c r="A32" s="47"/>
-      <c r="B32" s="48"/>
-      <c r="C32" s="49">
+      <c r="A32" s="44"/>
+      <c r="B32" s="45"/>
+      <c r="C32" s="46">
         <f>SUM(D2:D31)</f>
         <v>0</v>
       </c>
-      <c r="D32" s="50"/>
-      <c r="E32" s="51"/>
+      <c r="D32" s="47"/>
+      <c r="E32" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2873,14 +2939,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="21.1428571428571" style="13" customWidth="1"/>
-    <col min="2" max="2" width="37.8571428571429" style="12" customWidth="1"/>
-    <col min="3" max="3" width="30.752380952381" style="12" customWidth="1"/>
-    <col min="4" max="4" width="65.7047619047619" style="12" customWidth="1"/>
-    <col min="5" max="7" width="32.3333333333333" style="12" customWidth="1"/>
-    <col min="8" max="16384" width="9.14285714285714" style="12"/>
+    <col min="1" max="1" width="21.140625" style="13" customWidth="1"/>
+    <col min="2" max="2" width="37.859375" style="12" customWidth="1"/>
+    <col min="3" max="3" width="30.75" style="12" customWidth="1"/>
+    <col min="4" max="4" width="65.703125" style="12" customWidth="1"/>
+    <col min="5" max="7" width="32.3359375" style="12" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="12"/>
   </cols>
   <sheetData>
     <row r="1" s="11" customFormat="1" ht="35" customHeight="1" spans="1:7">
@@ -2888,10 +2954,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D1" s="15" t="s">
         <v>4</v>
@@ -2911,147 +2977,147 @@
         <v>45992</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C2" s="18">
         <v>1</v>
       </c>
       <c r="D2" s="19"/>
-      <c r="E2" s="20">
+      <c r="E2" s="29">
         <v>60000</v>
       </c>
-      <c r="F2" s="21">
-        <f>C2*E2</f>
+      <c r="F2" s="30">
+        <f t="shared" ref="F2:F8" si="0">C2*E2</f>
         <v>60000</v>
       </c>
-      <c r="G2" s="22">
+      <c r="G2" s="31">
         <f>SUM(F2:F3)</f>
         <v>115000</v>
       </c>
     </row>
     <row r="3" s="12" customFormat="1" ht="80" customHeight="1" spans="1:7">
-      <c r="A3" s="23"/>
-      <c r="B3" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3" s="25">
+      <c r="A3" s="20"/>
+      <c r="B3" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="22">
         <v>1</v>
       </c>
-      <c r="D3" s="26"/>
-      <c r="E3" s="20">
+      <c r="D3" s="23"/>
+      <c r="E3" s="29">
         <v>55000</v>
       </c>
-      <c r="F3" s="21">
-        <f>C3*E3</f>
+      <c r="F3" s="30">
+        <f t="shared" si="0"/>
         <v>55000</v>
       </c>
-      <c r="G3" s="22"/>
+      <c r="G3" s="31"/>
     </row>
     <row r="4" s="12" customFormat="1" ht="48" customHeight="1" spans="1:7">
-      <c r="A4" s="27">
+      <c r="A4" s="24">
         <v>46003</v>
       </c>
-      <c r="B4" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="25">
+      <c r="B4" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="22">
         <v>3</v>
       </c>
-      <c r="D4" s="28"/>
-      <c r="E4" s="20">
+      <c r="D4" s="25"/>
+      <c r="E4" s="29">
         <v>55000</v>
       </c>
-      <c r="F4" s="21">
-        <f>C4*E4</f>
+      <c r="F4" s="30">
+        <f t="shared" si="0"/>
         <v>165000</v>
       </c>
-      <c r="G4" s="29">
+      <c r="G4" s="32">
         <f>SUM(F4:F8)</f>
         <v>735000</v>
       </c>
     </row>
     <row r="5" s="12" customFormat="1" ht="48" customHeight="1" spans="1:7">
-      <c r="A5" s="30"/>
-      <c r="B5" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="25">
+      <c r="A5" s="26"/>
+      <c r="B5" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="22">
         <v>1</v>
       </c>
-      <c r="D5" s="28"/>
-      <c r="E5" s="20">
+      <c r="D5" s="25"/>
+      <c r="E5" s="29">
         <v>160000</v>
       </c>
-      <c r="F5" s="21">
-        <f>C5*E5</f>
+      <c r="F5" s="30">
+        <f t="shared" si="0"/>
         <v>160000</v>
       </c>
-      <c r="G5" s="29"/>
+      <c r="G5" s="32"/>
     </row>
     <row r="6" s="12" customFormat="1" ht="48" customHeight="1" spans="1:7">
-      <c r="A6" s="30"/>
-      <c r="B6" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="25">
+      <c r="A6" s="26"/>
+      <c r="B6" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="22">
         <v>1</v>
       </c>
-      <c r="D6" s="28"/>
-      <c r="E6" s="20">
+      <c r="D6" s="25"/>
+      <c r="E6" s="29">
         <v>60000</v>
       </c>
-      <c r="F6" s="21">
-        <f>C6*E6</f>
+      <c r="F6" s="30">
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
-      <c r="G6" s="29"/>
+      <c r="G6" s="32"/>
     </row>
     <row r="7" s="12" customFormat="1" ht="48" customHeight="1" spans="1:7">
-      <c r="A7" s="30"/>
-      <c r="B7" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="25">
+      <c r="A7" s="26"/>
+      <c r="B7" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="22">
         <v>3</v>
       </c>
-      <c r="D7" s="28"/>
-      <c r="E7" s="20">
+      <c r="D7" s="25"/>
+      <c r="E7" s="29">
         <v>50000</v>
       </c>
-      <c r="F7" s="21">
-        <f>C7*E7</f>
+      <c r="F7" s="30">
+        <f t="shared" si="0"/>
         <v>150000</v>
       </c>
-      <c r="G7" s="29"/>
+      <c r="G7" s="32"/>
     </row>
     <row r="8" s="12" customFormat="1" ht="48" customHeight="1" spans="1:7">
-      <c r="A8" s="31"/>
-      <c r="B8" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" s="25">
+      <c r="A8" s="27"/>
+      <c r="B8" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="22">
         <v>1</v>
       </c>
-      <c r="D8" s="28"/>
-      <c r="E8" s="20">
+      <c r="D8" s="25"/>
+      <c r="E8" s="29">
         <v>200000</v>
       </c>
-      <c r="F8" s="21">
-        <f>C8*E8</f>
+      <c r="F8" s="30">
+        <f t="shared" si="0"/>
         <v>200000</v>
       </c>
-      <c r="G8" s="32"/>
+      <c r="G8" s="33"/>
     </row>
     <row r="9" s="12" customFormat="1" ht="39" customHeight="1" spans="1:7">
-      <c r="A9" s="33" t="s">
+      <c r="A9" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="34"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="36">
+      <c r="B9" s="25"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="34">
         <f>SUM(G2:G8)</f>
         <v>850000</v>
       </c>
@@ -3075,22 +3141,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelRow="6" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="9.14285714285714" style="1"/>
-    <col min="2" max="2" width="21.8571428571429" style="2" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
+    <col min="2" max="2" width="21.859375" style="2" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:3">
       <c r="A1" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -3098,7 +3164,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C2" s="8">
         <f>'Anugrah (Bag, Cup, Box)'!H9</f>
@@ -3110,11 +3176,11 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C3" s="8">
-        <f>'UD Abdi Jaya (Bag, Cup, Box)'!H11</f>
-        <v>4197500</v>
+        <f>'UD Abdi Jaya (Bag, Cup, Box)'!H12</f>
+        <v>5945000</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -3122,7 +3188,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C4" s="8">
         <f>'PT. SUPARMA JAYA TBK (Tissue)'!E14</f>
@@ -3134,7 +3200,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C5" s="9">
         <f>'Vickel Laundry'!C32</f>
@@ -3146,7 +3212,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C6" s="9">
         <f>'Dishy Soap'!G9</f>
@@ -3160,7 +3226,7 @@
       <c r="B7" s="7"/>
       <c r="C7" s="10">
         <f>SUM(C2:C5)</f>
-        <v>6094500</v>
+        <v>7842000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2 JAN 2025 14:14
</commit_message>
<xml_diff>
--- a/DECEMBER/DECEMBER FLOOR.xlsx
+++ b/DECEMBER/DECEMBER FLOOR.xlsx
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="49">
   <si>
     <t>DATE</t>
   </si>
@@ -126,6 +126,12 @@
   </si>
   <si>
     <t>CUP HOLDER DOUBLE</t>
+  </si>
+  <si>
+    <t>CUP INJECTION 400 ML</t>
+  </si>
+  <si>
+    <t>PAPER BAG CB 7</t>
   </si>
   <si>
     <t>0608</t>
@@ -1071,7 +1077,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="136">
+  <cellXfs count="148">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1371,18 +1377,24 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="182" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1392,22 +1404,31 @@
     <xf numFmtId="183" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="183" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="183" fontId="9" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="11" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="11" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="11" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1417,6 +1438,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="9" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1425,9 +1449,18 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="181" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="180" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1438,6 +1471,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1569,53 +1611,14 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>22542</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>33972</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>3913822</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>336867</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="ID_EA4BA6ECE5B54036826B94B9F6D867FF" descr="WhatsApp Image 2025-12-11 at 18.49.57_9a9d137a"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:srcRect t="13770" b="11839"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm rot="16200000">
-          <a:off x="8345170" y="2624455"/>
-          <a:ext cx="2880995" cy="3891280"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
       <xdr:colOff>30797</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>15</xdr:row>
       <xdr:rowOff>26987</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>4770437</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>15</xdr:row>
       <xdr:rowOff>4471352</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1626,7 +1629,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
+        <a:blip r:embed="rId2"/>
         <a:srcRect l="2346" t="14598" b="17958"/>
         <a:stretch>
           <a:fillRect/>
@@ -1634,7 +1637,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm rot="16200000">
-          <a:off x="7995920" y="5921375"/>
+          <a:off x="7995920" y="10188575"/>
           <a:ext cx="4444365" cy="4739640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1648,13 +1651,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>35560</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>27940</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>4766310</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>3897630</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1665,7 +1668,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId4"/>
+        <a:blip r:embed="rId3"/>
         <a:srcRect t="19236" b="11470"/>
         <a:stretch>
           <a:fillRect/>
@@ -1673,12 +1676,98 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm rot="16200000">
-          <a:off x="8284210" y="10134600"/>
+          <a:off x="8284210" y="14401800"/>
           <a:ext cx="3869690" cy="4730750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>46672</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>26987</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>4754562</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>873442</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="ID_FC0423A889E649A690042F7E81C03532"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:srcRect t="25750" r="2659" b="15363"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="8461375" y="6182995"/>
+          <a:ext cx="3513455" cy="4707890"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>88265</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>29845</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>4713605</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>386715</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="ID_DD8F384FE1394649869746B752992DB5"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId5"/>
+        <a:srcRect t="26542" b="15720"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="8415020" y="2617470"/>
+          <a:ext cx="3608070" cy="4625340"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -2082,161 +2171,161 @@
   </cols>
   <sheetData>
     <row r="1" s="88" customFormat="1" ht="16" customHeight="1" spans="1:8">
-      <c r="A1" s="121" t="s">
+      <c r="A1" s="126" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="122" t="s">
+      <c r="B1" s="127" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="122" t="s">
+      <c r="C1" s="127" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="122" t="s">
+      <c r="D1" s="127" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="122" t="s">
+      <c r="E1" s="127" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="122" t="s">
+      <c r="F1" s="127" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="122" t="s">
+      <c r="G1" s="127" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="122" t="s">
+      <c r="H1" s="127" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" s="88" customFormat="1" ht="120" customHeight="1" spans="1:8">
-      <c r="A2" s="99">
+      <c r="A2" s="128">
         <v>45994</v>
       </c>
       <c r="B2" s="96">
         <v>2518</v>
       </c>
-      <c r="C2" s="123" t="s">
+      <c r="C2" s="129" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="124">
+      <c r="D2" s="130">
         <v>4</v>
       </c>
-      <c r="E2" s="111" t="str">
+      <c r="E2" s="113" t="str">
         <f>_xlfn.DISPIMG("ID_AF642E9448564DC2B9A94250BEBF50D7",1)</f>
         <v>=DISPIMG("ID_AF642E9448564DC2B9A94250BEBF50D7",1)</v>
       </c>
-      <c r="F2" s="112">
+      <c r="F2" s="114">
         <v>178000</v>
       </c>
-      <c r="G2" s="114">
+      <c r="G2" s="139">
         <f t="shared" ref="G2:G8" si="0">SUM(D2*F2)</f>
         <v>712000</v>
       </c>
-      <c r="H2" s="114">
+      <c r="H2" s="139">
         <f>SUM(G2:G3)</f>
         <v>1897000</v>
       </c>
     </row>
     <row r="3" s="88" customFormat="1" ht="120" customHeight="1" spans="1:8">
-      <c r="A3" s="102"/>
+      <c r="A3" s="131"/>
       <c r="B3" s="96"/>
-      <c r="C3" s="123" t="s">
+      <c r="C3" s="129" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="124">
+      <c r="D3" s="130">
         <v>3</v>
       </c>
-      <c r="E3" s="115"/>
-      <c r="F3" s="112">
+      <c r="E3" s="140"/>
+      <c r="F3" s="114">
         <v>395000</v>
       </c>
-      <c r="G3" s="114">
+      <c r="G3" s="139">
         <f t="shared" si="0"/>
         <v>1185000</v>
       </c>
-      <c r="H3" s="116"/>
+      <c r="H3" s="141"/>
     </row>
     <row r="4" s="88" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A4" s="99"/>
-      <c r="B4" s="100"/>
-      <c r="C4" s="125"/>
-      <c r="D4" s="124"/>
-      <c r="E4" s="111"/>
-      <c r="F4" s="114"/>
-      <c r="G4" s="114">
+      <c r="A4" s="128"/>
+      <c r="B4" s="132"/>
+      <c r="C4" s="133"/>
+      <c r="D4" s="130"/>
+      <c r="E4" s="113"/>
+      <c r="F4" s="139"/>
+      <c r="G4" s="139">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H4" s="114">
+      <c r="H4" s="139">
         <f>SUM(G4:G7)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" s="88" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A5" s="102"/>
-      <c r="B5" s="103"/>
+      <c r="A5" s="131"/>
+      <c r="B5" s="134"/>
       <c r="C5" s="96"/>
       <c r="D5" s="96"/>
-      <c r="E5" s="115"/>
-      <c r="F5" s="130"/>
-      <c r="G5" s="114">
+      <c r="E5" s="140"/>
+      <c r="F5" s="142"/>
+      <c r="G5" s="139">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H5" s="116"/>
+      <c r="H5" s="141"/>
     </row>
     <row r="6" s="88" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A6" s="102"/>
-      <c r="B6" s="103"/>
+      <c r="A6" s="131"/>
+      <c r="B6" s="134"/>
       <c r="C6" s="96"/>
       <c r="D6" s="96"/>
-      <c r="E6" s="115"/>
-      <c r="F6" s="130"/>
-      <c r="G6" s="114">
+      <c r="E6" s="140"/>
+      <c r="F6" s="142"/>
+      <c r="G6" s="139">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="116"/>
+      <c r="H6" s="141"/>
     </row>
     <row r="7" s="88" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A7" s="102"/>
-      <c r="B7" s="103"/>
-      <c r="C7" s="100"/>
-      <c r="D7" s="100"/>
-      <c r="E7" s="115"/>
-      <c r="F7" s="130"/>
-      <c r="G7" s="114">
+      <c r="A7" s="131"/>
+      <c r="B7" s="134"/>
+      <c r="C7" s="132"/>
+      <c r="D7" s="132"/>
+      <c r="E7" s="140"/>
+      <c r="F7" s="142"/>
+      <c r="G7" s="139">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H7" s="116"/>
+      <c r="H7" s="141"/>
     </row>
     <row r="8" s="88" customFormat="1" ht="258" customHeight="1" spans="1:8">
       <c r="A8" s="95"/>
       <c r="B8" s="96"/>
       <c r="C8" s="96"/>
       <c r="D8" s="96"/>
-      <c r="E8" s="131"/>
-      <c r="F8" s="132"/>
-      <c r="G8" s="112">
+      <c r="E8" s="143"/>
+      <c r="F8" s="144"/>
+      <c r="G8" s="114">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="112">
+      <c r="H8" s="114">
         <f>SUM(G8)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" s="88" customFormat="1" ht="18" customHeight="1" spans="1:8">
-      <c r="A9" s="126" t="s">
+      <c r="A9" s="135" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="127"/>
-      <c r="C9" s="128"/>
-      <c r="D9" s="129"/>
-      <c r="E9" s="133"/>
-      <c r="F9" s="133"/>
-      <c r="G9" s="134"/>
-      <c r="H9" s="135">
+      <c r="B9" s="136"/>
+      <c r="C9" s="137"/>
+      <c r="D9" s="138"/>
+      <c r="E9" s="145"/>
+      <c r="F9" s="145"/>
+      <c r="G9" s="146"/>
+      <c r="H9" s="147">
         <f>SUM(H2:H8)</f>
         <v>1897000</v>
       </c>
@@ -2261,7 +2350,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="20.4" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="19.859375" style="89"/>
@@ -2314,24 +2403,24 @@
       <c r="D2" s="98">
         <v>3</v>
       </c>
-      <c r="E2" s="111"/>
-      <c r="F2" s="112">
+      <c r="E2" s="113"/>
+      <c r="F2" s="114">
         <v>55000</v>
       </c>
-      <c r="G2" s="113">
+      <c r="G2" s="115">
         <f t="shared" ref="G2:G12" si="0">D2*F2</f>
         <v>165000</v>
       </c>
-      <c r="H2" s="112">
+      <c r="H2" s="116">
         <f>SUM(G2:G2)</f>
         <v>165000</v>
       </c>
     </row>
-    <row r="3" s="88" customFormat="1" ht="29" customHeight="1" spans="1:8">
+    <row r="3" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
       <c r="A3" s="99">
         <v>46002</v>
       </c>
-      <c r="B3" s="136" t="s">
+      <c r="B3" s="148" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="101" t="s">
@@ -2340,20 +2429,20 @@
       <c r="D3" s="98">
         <v>1</v>
       </c>
-      <c r="E3" s="111"/>
-      <c r="F3" s="113">
+      <c r="E3" s="117"/>
+      <c r="F3" s="115">
         <v>295000</v>
       </c>
-      <c r="G3" s="113">
+      <c r="G3" s="115">
         <f t="shared" si="0"/>
         <v>295000</v>
       </c>
-      <c r="H3" s="114">
-        <f>SUM(G3:G10)</f>
-        <v>5280000</v>
-      </c>
-    </row>
-    <row r="4" s="88" customFormat="1" ht="29" customHeight="1" spans="1:8">
+      <c r="H3" s="118">
+        <f>SUM(G3:G11)</f>
+        <v>5630000</v>
+      </c>
+    </row>
+    <row r="4" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
       <c r="A4" s="102"/>
       <c r="B4" s="103"/>
       <c r="C4" s="101" t="s">
@@ -2362,17 +2451,17 @@
       <c r="D4" s="98">
         <v>4</v>
       </c>
-      <c r="E4" s="115"/>
-      <c r="F4" s="113">
+      <c r="E4" s="119"/>
+      <c r="F4" s="115">
         <v>150000</v>
       </c>
-      <c r="G4" s="113">
+      <c r="G4" s="115">
         <f t="shared" si="0"/>
         <v>600000</v>
       </c>
-      <c r="H4" s="116"/>
-    </row>
-    <row r="5" s="88" customFormat="1" ht="29" customHeight="1" spans="1:8">
+      <c r="H4" s="120"/>
+    </row>
+    <row r="5" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
       <c r="A5" s="102"/>
       <c r="B5" s="103"/>
       <c r="C5" s="101" t="s">
@@ -2381,17 +2470,17 @@
       <c r="D5" s="98">
         <v>4</v>
       </c>
-      <c r="E5" s="115"/>
-      <c r="F5" s="113">
+      <c r="E5" s="119"/>
+      <c r="F5" s="115">
         <v>460000</v>
       </c>
-      <c r="G5" s="113">
+      <c r="G5" s="115">
         <f t="shared" si="0"/>
         <v>1840000</v>
       </c>
-      <c r="H5" s="116"/>
-    </row>
-    <row r="6" s="88" customFormat="1" ht="29" customHeight="1" spans="1:8">
+      <c r="H5" s="120"/>
+    </row>
+    <row r="6" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
       <c r="A6" s="102"/>
       <c r="B6" s="103"/>
       <c r="C6" s="101" t="s">
@@ -2400,17 +2489,17 @@
       <c r="D6" s="98">
         <v>2</v>
       </c>
-      <c r="E6" s="115"/>
-      <c r="F6" s="113">
+      <c r="E6" s="119"/>
+      <c r="F6" s="115">
         <v>340000</v>
       </c>
-      <c r="G6" s="113">
+      <c r="G6" s="115">
         <f t="shared" si="0"/>
         <v>680000</v>
       </c>
-      <c r="H6" s="116"/>
-    </row>
-    <row r="7" s="88" customFormat="1" ht="29" customHeight="1" spans="1:8">
+      <c r="H6" s="120"/>
+    </row>
+    <row r="7" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
       <c r="A7" s="102"/>
       <c r="B7" s="103"/>
       <c r="C7" s="101" t="s">
@@ -2419,17 +2508,17 @@
       <c r="D7" s="98">
         <v>1</v>
       </c>
-      <c r="E7" s="115"/>
-      <c r="F7" s="112">
+      <c r="E7" s="119"/>
+      <c r="F7" s="114">
         <v>340000</v>
       </c>
-      <c r="G7" s="113">
+      <c r="G7" s="115">
         <f t="shared" si="0"/>
         <v>340000</v>
       </c>
-      <c r="H7" s="116"/>
-    </row>
-    <row r="8" s="88" customFormat="1" ht="29" customHeight="1" spans="1:8">
+      <c r="H7" s="120"/>
+    </row>
+    <row r="8" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
       <c r="A8" s="102"/>
       <c r="B8" s="103"/>
       <c r="C8" s="104" t="s">
@@ -2438,17 +2527,17 @@
       <c r="D8" s="96">
         <v>5</v>
       </c>
-      <c r="E8" s="115"/>
-      <c r="F8" s="96">
+      <c r="E8" s="119"/>
+      <c r="F8" s="114">
         <v>55000</v>
       </c>
-      <c r="G8" s="113">
+      <c r="G8" s="115">
         <f t="shared" si="0"/>
         <v>275000</v>
       </c>
-      <c r="H8" s="116"/>
-    </row>
-    <row r="9" s="88" customFormat="1" ht="29" customHeight="1" spans="1:8">
+      <c r="H8" s="120"/>
+    </row>
+    <row r="9" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
       <c r="A9" s="102"/>
       <c r="B9" s="103"/>
       <c r="C9" s="104" t="s">
@@ -2457,107 +2546,213 @@
       <c r="D9" s="96">
         <v>500</v>
       </c>
-      <c r="E9" s="115"/>
-      <c r="F9" s="96">
+      <c r="E9" s="119"/>
+      <c r="F9" s="114">
         <v>1000</v>
       </c>
-      <c r="G9" s="113">
+      <c r="G9" s="115">
         <f t="shared" si="0"/>
         <v>500000</v>
       </c>
-      <c r="H9" s="116"/>
-    </row>
-    <row r="10" s="88" customFormat="1" ht="29" customHeight="1" spans="1:8">
-      <c r="A10" s="105"/>
-      <c r="B10" s="106"/>
+      <c r="H9" s="120"/>
+    </row>
+    <row r="10" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
+      <c r="A10" s="102"/>
+      <c r="B10" s="103"/>
       <c r="C10" s="104" t="s">
         <v>20</v>
       </c>
       <c r="D10" s="96">
         <v>500</v>
       </c>
-      <c r="E10" s="117"/>
-      <c r="F10" s="96">
+      <c r="E10" s="119"/>
+      <c r="F10" s="114">
         <v>1500</v>
       </c>
-      <c r="G10" s="113">
+      <c r="G10" s="115">
         <f t="shared" si="0"/>
         <v>750000</v>
       </c>
-      <c r="H10" s="118"/>
-    </row>
-    <row r="11" s="88" customFormat="1" ht="353.9" customHeight="1" spans="1:8">
-      <c r="A11" s="107">
+      <c r="H10" s="120"/>
+    </row>
+    <row r="11" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
+      <c r="A11" s="105"/>
+      <c r="B11" s="106"/>
+      <c r="C11" s="107" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="108">
+        <v>10</v>
+      </c>
+      <c r="E11" s="121"/>
+      <c r="F11" s="114">
+        <v>35000</v>
+      </c>
+      <c r="G11" s="115">
+        <f>D11*F11</f>
+        <v>350000</v>
+      </c>
+      <c r="H11" s="120"/>
+    </row>
+    <row r="12" s="88" customFormat="1" ht="70" customHeight="1" spans="1:8">
+      <c r="A12" s="109">
+        <v>46003</v>
+      </c>
+      <c r="B12" s="110">
+        <v>938</v>
+      </c>
+      <c r="C12" s="107" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" s="108">
+        <v>4</v>
+      </c>
+      <c r="E12" s="110"/>
+      <c r="F12" s="114">
+        <v>500000</v>
+      </c>
+      <c r="G12" s="115">
+        <f>D12*F12</f>
+        <v>2000000</v>
+      </c>
+      <c r="H12" s="122">
+        <f>SUM(G12:G15)</f>
+        <v>2740000</v>
+      </c>
+    </row>
+    <row r="13" s="88" customFormat="1" ht="70" customHeight="1" spans="1:8">
+      <c r="A13" s="109"/>
+      <c r="B13" s="110"/>
+      <c r="C13" s="107" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="108">
+        <v>1</v>
+      </c>
+      <c r="E13" s="110"/>
+      <c r="F13" s="114">
+        <v>340000</v>
+      </c>
+      <c r="G13" s="115">
+        <f>D13*F13</f>
+        <v>340000</v>
+      </c>
+      <c r="H13" s="122"/>
+    </row>
+    <row r="14" s="88" customFormat="1" ht="70" customHeight="1" spans="1:8">
+      <c r="A14" s="109"/>
+      <c r="B14" s="110"/>
+      <c r="C14" s="107" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="108">
+        <v>2</v>
+      </c>
+      <c r="E14" s="110"/>
+      <c r="F14" s="114">
+        <v>25000</v>
+      </c>
+      <c r="G14" s="115">
+        <f>D14*F14</f>
+        <v>50000</v>
+      </c>
+      <c r="H14" s="122"/>
+    </row>
+    <row r="15" s="88" customFormat="1" ht="70" customHeight="1" spans="1:8">
+      <c r="A15" s="109"/>
+      <c r="B15" s="110"/>
+      <c r="C15" s="107" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="108">
+        <v>10</v>
+      </c>
+      <c r="E15" s="110"/>
+      <c r="F15" s="114">
+        <v>35000</v>
+      </c>
+      <c r="G15" s="115">
+        <f>D15*F15</f>
+        <v>350000</v>
+      </c>
+      <c r="H15" s="123"/>
+    </row>
+    <row r="16" s="88" customFormat="1" ht="353.9" customHeight="1" spans="1:8">
+      <c r="A16" s="111">
         <v>46008</v>
       </c>
-      <c r="B11" s="137" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="109" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="110">
+      <c r="B16" s="149" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="107" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="108">
         <v>20</v>
       </c>
-      <c r="E11" s="108"/>
-      <c r="F11" s="110">
+      <c r="E16" s="112"/>
+      <c r="F16" s="108">
         <v>25000</v>
       </c>
-      <c r="G11" s="113">
-        <f t="shared" si="0"/>
+      <c r="G16" s="115">
+        <f>D16*F16</f>
         <v>500000</v>
       </c>
-      <c r="H11" s="119">
-        <f>SUM(G11)</f>
+      <c r="H16" s="124">
+        <f>SUM(G16)</f>
         <v>500000</v>
       </c>
     </row>
-    <row r="12" s="88" customFormat="1" ht="308.9" customHeight="1" spans="1:8">
-      <c r="A12" s="107">
+    <row r="17" s="88" customFormat="1" ht="308.9" customHeight="1" spans="1:8">
+      <c r="A17" s="111">
         <v>46013</v>
       </c>
-      <c r="B12" s="137" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="109" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="110">
+      <c r="B17" s="149" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="107" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17" s="108">
         <v>10</v>
       </c>
-      <c r="E12" s="108"/>
-      <c r="F12" s="110">
+      <c r="E17" s="112"/>
+      <c r="F17" s="108">
         <v>35000</v>
       </c>
-      <c r="G12" s="113">
-        <f t="shared" si="0"/>
+      <c r="G17" s="115">
+        <f>D17*F17</f>
         <v>350000</v>
       </c>
-      <c r="H12" s="119">
-        <f>SUM(G12)</f>
+      <c r="H17" s="124">
+        <f>SUM(G17)</f>
         <v>350000</v>
       </c>
     </row>
-    <row r="13" s="88" customFormat="1" spans="1:8">
-      <c r="A13" s="110"/>
-      <c r="B13" s="110"/>
-      <c r="C13" s="109"/>
-      <c r="D13" s="110"/>
-      <c r="E13" s="110"/>
-      <c r="F13" s="110"/>
-      <c r="G13" s="113"/>
-      <c r="H13" s="120">
-        <f>SUM(H2:H12)</f>
-        <v>6295000</v>
+    <row r="18" s="88" customFormat="1" spans="1:8">
+      <c r="A18" s="108"/>
+      <c r="B18" s="108"/>
+      <c r="C18" s="107"/>
+      <c r="D18" s="108"/>
+      <c r="E18" s="108"/>
+      <c r="F18" s="108"/>
+      <c r="G18" s="115"/>
+      <c r="H18" s="125">
+        <f>SUM(H2:H17)</f>
+        <v>9385000</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A3:A10"/>
-    <mergeCell ref="B3:B10"/>
-    <mergeCell ref="E3:E10"/>
-    <mergeCell ref="H3:H10"/>
+  <mergeCells count="9">
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A3:A11"/>
+    <mergeCell ref="A12:A15"/>
+    <mergeCell ref="B3:B11"/>
+    <mergeCell ref="B12:B15"/>
+    <mergeCell ref="E3:E11"/>
+    <mergeCell ref="E12:E15"/>
+    <mergeCell ref="H3:H11"/>
+    <mergeCell ref="H12:H15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -2627,7 +2822,7 @@
     <row r="4" spans="1:7">
       <c r="A4" s="53"/>
       <c r="B4" s="58" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="58"/>
       <c r="D4" s="59"/>
@@ -2641,7 +2836,7 @@
     <row r="5" spans="1:7">
       <c r="A5" s="53"/>
       <c r="B5" s="58" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" s="58"/>
       <c r="D5" s="59"/>
@@ -2655,7 +2850,7 @@
     <row r="6" spans="1:7">
       <c r="A6" s="53"/>
       <c r="B6" s="58" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C6" s="58"/>
       <c r="D6" s="59"/>
@@ -2697,7 +2892,7 @@
     <row r="10" spans="1:7">
       <c r="A10" s="64"/>
       <c r="B10" s="58" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C10" s="58"/>
       <c r="D10" s="59"/>
@@ -2711,7 +2906,7 @@
     <row r="11" spans="1:7">
       <c r="A11" s="65"/>
       <c r="B11" s="66" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C11" s="67"/>
       <c r="D11" s="59"/>
@@ -2722,7 +2917,7 @@
     <row r="12" spans="1:7">
       <c r="A12" s="64"/>
       <c r="B12" s="58" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C12" s="58"/>
       <c r="D12" s="59"/>
@@ -2814,7 +3009,7 @@
         <v>7</v>
       </c>
       <c r="E1" s="38" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" s="12" customFormat="1" ht="263.65" customHeight="1" spans="1:5">
@@ -3070,10 +3265,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D1" s="15" t="s">
         <v>4</v>
@@ -3093,7 +3288,7 @@
         <v>45992</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C2" s="18">
         <v>1</v>
@@ -3114,7 +3309,7 @@
     <row r="3" s="12" customFormat="1" ht="80" customHeight="1" spans="1:7">
       <c r="A3" s="20"/>
       <c r="B3" s="21" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C3" s="22">
         <v>1</v>
@@ -3134,7 +3329,7 @@
         <v>46003</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C4" s="22">
         <v>3</v>
@@ -3155,7 +3350,7 @@
     <row r="5" s="12" customFormat="1" ht="48" customHeight="1" spans="1:7">
       <c r="A5" s="26"/>
       <c r="B5" s="21" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C5" s="22">
         <v>1</v>
@@ -3173,7 +3368,7 @@
     <row r="6" s="12" customFormat="1" ht="48" customHeight="1" spans="1:7">
       <c r="A6" s="26"/>
       <c r="B6" s="21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C6" s="22">
         <v>1</v>
@@ -3191,7 +3386,7 @@
     <row r="7" s="12" customFormat="1" ht="48" customHeight="1" spans="1:7">
       <c r="A7" s="26"/>
       <c r="B7" s="21" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C7" s="22">
         <v>3</v>
@@ -3209,7 +3404,7 @@
     <row r="8" s="12" customFormat="1" ht="48" customHeight="1" spans="1:7">
       <c r="A8" s="27"/>
       <c r="B8" s="21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C8" s="22">
         <v>1</v>
@@ -3229,7 +3424,7 @@
         <v>46013</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C9" s="22">
         <v>3</v>
@@ -3289,13 +3484,13 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:3">
       <c r="A1" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -3303,7 +3498,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C2" s="8">
         <f>'Anugrah (Bag, Cup, Box)'!H9</f>
@@ -3315,11 +3510,11 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C3" s="8">
-        <f>'UD Abdi Jaya (Bag, Cup, Box)'!H13</f>
-        <v>6295000</v>
+        <f>'UD Abdi Jaya (Bag, Cup, Box)'!H18</f>
+        <v>9385000</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -3327,7 +3522,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C4" s="8">
         <f>'PT. SUPARMA JAYA TBK (Tissue)'!E14</f>
@@ -3339,7 +3534,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C5" s="9">
         <f>'Vickel Laundry'!C32</f>
@@ -3351,7 +3546,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C6" s="9">
         <f>'Dishy Soap'!G10</f>
@@ -3365,7 +3560,7 @@
       <c r="B7" s="7"/>
       <c r="C7" s="10">
         <f>SUM(C2:C5)</f>
-        <v>8192000</v>
+        <v>11282000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
3 jan 2026 16.26
</commit_message>
<xml_diff>
--- a/DECEMBER/DECEMBER FLOOR.xlsx
+++ b/DECEMBER/DECEMBER FLOOR.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17020" activeTab="1"/>
+    <workbookView windowHeight="16060" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Anugrah (Bag, Cup, Box)" sheetId="1" r:id="rId1"/>
@@ -59,11 +59,123 @@
       </xdr:spPr>
     </xdr:pic>
   </etc:cellImage>
+  <etc:cellImage>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="ID_6BB72733B67442EAB4426B445D61C75A"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:srcRect t="25750" r="2659" b="15363"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="8461375" y="3289935"/>
+          <a:ext cx="3513455" cy="4707890"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+  </etc:cellImage>
+  <etc:cellImage>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="ID_8F95A6AC7B8A4D948EAF5FC4A9DACCAC" descr="PHOTO-2025-12-22-19-55-17"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:srcRect t="19236" b="11470"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="8284210" y="11508740"/>
+          <a:ext cx="3869690" cy="4730750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+  </etc:cellImage>
+  <etc:cellImage>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="ID_360A81D236BB40E99ADBAD1BA0483D4A" descr="PHOTO-2025-12-17-17-40-21"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:srcRect l="2346" t="14598" b="17958"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="7995920" y="7295515"/>
+          <a:ext cx="4444365" cy="4739640"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+  </etc:cellImage>
+  <etc:cellImage>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="ID_515301B36E6F4ABA90C3BE145E0FA8EF"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId5"/>
+        <a:srcRect t="26542" b="15720"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="8415020" y="-275590"/>
+          <a:ext cx="3608070" cy="4625340"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+  </etc:cellImage>
 </etc:cellImages>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="61">
   <si>
     <t>DATE</t>
   </si>
@@ -98,7 +210,7 @@
     <t>GRAND TOTAL</t>
   </si>
   <si>
-    <t>HAND GLOVES (M)</t>
+    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t>0414</t>
@@ -155,7 +267,43 @@
     <t>PPh 22</t>
   </si>
   <si>
-    <t>STATUS</t>
+    <t>WEIGHT</t>
+  </si>
+  <si>
+    <t>0889</t>
+  </si>
+  <si>
+    <t>0890</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>0891</t>
+  </si>
+  <si>
+    <t>0892</t>
+  </si>
+  <si>
+    <t>0893</t>
+  </si>
+  <si>
+    <t>0894</t>
+  </si>
+  <si>
+    <t>0895</t>
+  </si>
+  <si>
+    <t>0896</t>
+  </si>
+  <si>
+    <t>0898</t>
+  </si>
+  <si>
+    <t>0899</t>
+  </si>
+  <si>
+    <t>0900</t>
   </si>
   <si>
     <t>DESCRIPTION</t>
@@ -216,17 +364,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="10">
+  <numFmts count="13">
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="180" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="181" formatCode="[$-409]d\-mmm\-yyyy;@"/>
-    <numFmt numFmtId="182" formatCode="dd\-mmm"/>
-    <numFmt numFmtId="183" formatCode="_ [$IDR]\ * #,##0_ ;_ [$IDR]\ * \-#,##0_ ;_ [$IDR]\ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="184" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="185" formatCode="_-&quot;Rp&quot;* #,##0.00_-;\-&quot;Rp&quot;* #,##0.00_-;_-&quot;Rp&quot;* &quot;-&quot;??.00_-;_-@_-"/>
+    <numFmt numFmtId="182" formatCode="0.00_);[Red]\(0.00\)"/>
+    <numFmt numFmtId="183" formatCode="[$Rp-421]#,##0.00_);[Red]\([$Rp-421]#,##0.00\)"/>
+    <numFmt numFmtId="184" formatCode="dd\-mmm"/>
+    <numFmt numFmtId="185" formatCode="0.0_);[Red]\(0.0\)"/>
+    <numFmt numFmtId="186" formatCode="_ [$IDR]\ * #,##0_ ;_ [$IDR]\ * \-#,##0_ ;_ [$IDR]\ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="187" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="188" formatCode="_-&quot;Rp&quot;* #,##0.00_-;\-&quot;Rp&quot;* #,##0.00_-;_-&quot;Rp&quot;* &quot;-&quot;??.00_-;_-@_-"/>
   </numFmts>
   <fonts count="33">
     <font>
@@ -799,17 +950,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color auto="1"/>
       </left>
@@ -826,6 +966,17 @@
         <color auto="1"/>
       </right>
       <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -1077,7 +1228,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="148">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1184,20 +1335,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="184" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="185" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="183" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1205,23 +1368,14 @@
     <xf numFmtId="183" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1250,16 +1404,13 @@
     <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="182" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="184" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="184" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1271,16 +1422,16 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1289,23 +1440,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="184" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="183" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="185" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="186" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="187" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="186" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="188" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="184" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="186" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="187" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1318,7 +1472,7 @@
     <xf numFmtId="180" fontId="8" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1341,18 +1495,6 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="181" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1362,6 +1504,9 @@
     <xf numFmtId="180" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="181" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1371,6 +1516,9 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="181" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1383,13 +1531,13 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="184" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="184" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1398,25 +1546,19 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="183" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="183" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="183" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="186" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="186" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="9" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="186" fontId="10" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="186" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1438,9 +1580,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="9" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1449,22 +1588,16 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="180" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1473,13 +1606,10 @@
     <xf numFmtId="180" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="183" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="186" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="186" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1494,7 +1624,7 @@
     <xf numFmtId="180" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="186" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1504,6 +1634,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1571,243 +1704,35 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>31750</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>27305</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>43180</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>29210</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>3899535</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>2866390</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>5306060</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>3606800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="ID_9870CD9F67EF4A49AA830086E9844D26" descr="WhatsApp Image 2025-12-11 at 19.04.33_291d8f18"/>
+        <xdr:cNvPr id="8" name="ID_A223130C6D474ECEA68D87A558FBBD81" descr="PHOTO-2025-12-22-18-49-25"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip r:embed="rId1"/>
-        <a:srcRect t="11037" b="12496"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm rot="5400000">
-          <a:off x="8364220" y="-283845"/>
-          <a:ext cx="2839085" cy="3867785"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>30797</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>26987</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>4770437</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>4471352</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="ID_FDB04E1C200E40C2A01C8C6D07A45482" descr="PHOTO-2025-12-17-17-40-21"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:srcRect l="2346" t="14598" b="17958"/>
+        <a:srcRect l="8940" t="19039" r="7862" b="12149"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm rot="16200000">
-          <a:off x="7995920" y="10188575"/>
-          <a:ext cx="4444365" cy="4739640"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>35560</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>27940</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>4766310</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>3897630</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="ID_D86B1F4AC6B747339C3E09790F41C073" descr="PHOTO-2025-12-22-19-55-17"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:srcRect t="19236" b="11470"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm rot="16200000">
-          <a:off x="8284210" y="14401800"/>
-          <a:ext cx="3869690" cy="4730750"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>46672</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>26987</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>4754562</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>873442</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="ID_FC0423A889E649A690042F7E81C03532"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId4"/>
-        <a:srcRect t="25750" r="2659" b="15363"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm rot="16200000">
-          <a:off x="8461375" y="6182995"/>
-          <a:ext cx="3513455" cy="4707890"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>88265</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>29845</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>4713605</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>386715</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="ID_DD8F384FE1394649869746B752992DB5"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId5"/>
-        <a:srcRect t="26542" b="15720"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm rot="16200000">
-          <a:off x="8415020" y="2617470"/>
-          <a:ext cx="3608070" cy="4625340"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>26035</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>56515</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>4355465</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>949325</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="ID_7BEFDB63F16448A5BB21710E631EB358" descr="WhatsApp Image 2025-12-03 at 11.37.37_bfde9d0a"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:srcRect l="6138" t="14811" b="10638"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm rot="16200000">
-          <a:off x="7953375" y="-131445"/>
-          <a:ext cx="3064510" cy="4329430"/>
+          <a:off x="8180705" y="5866765"/>
+          <a:ext cx="3577590" cy="5262880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1819,19 +1744,19 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>19367</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>1011872</xdr:rowOff>
+      <xdr:colOff>520065</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>29210</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4348797</xdr:colOff>
+      <xdr:colOff>4829175</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>564197</xdr:rowOff>
+      <xdr:rowOff>582930</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="ID_F4D3B8AB0BD24917BF078073AEC51FE5" descr="WhatsApp Image 2025-12-12 at 12.56.20_53e90f5f"/>
+        <xdr:cNvPr id="7" name="ID_1DCF24B9869548A9BB648FC98316A878" descr="WhatsApp Image 2025-12-12 at 12.56.20_53e90f5f"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -1845,8 +1770,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm rot="16200000">
-          <a:off x="7974965" y="2966085"/>
-          <a:ext cx="3006725" cy="4329430"/>
+          <a:off x="8473440" y="3002915"/>
+          <a:ext cx="2992120" cy="4309110"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1858,34 +1783,34 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>43180</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>29210</xdr:rowOff>
+      <xdr:colOff>509905</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>61595</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>5306060</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>3606800</xdr:rowOff>
+      <xdr:colOff>4839335</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>954405</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="ID_62FF72CEF4C648BA90698309D9EEDEC4" descr="PHOTO-2025-12-22-18-49-25"/>
+        <xdr:cNvPr id="5" name="ID_A03A8F9AC41643A998951A68911C5346" descr="WhatsApp Image 2025-12-03 at 11.37.37_bfde9d0a"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip r:embed="rId3"/>
-        <a:srcRect l="8940" t="19039" r="7862" b="12149"/>
+        <a:srcRect l="6138" t="14811" b="10638"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm rot="16200000">
-          <a:off x="8180705" y="5866765"/>
-          <a:ext cx="3577590" cy="5262880"/>
+          <a:off x="8437245" y="-126365"/>
+          <a:ext cx="3064510" cy="4329430"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2158,174 +2083,174 @@
   <dimension ref="A1:H9"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="20.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="17.4296875" style="91"/>
-    <col min="2" max="2" width="13.4296875" style="91" customWidth="1"/>
-    <col min="3" max="3" width="36" style="91" customWidth="1"/>
-    <col min="4" max="4" width="21.2890625" style="89" customWidth="1"/>
-    <col min="5" max="5" width="33.2890625" style="91" customWidth="1"/>
-    <col min="6" max="6" width="17.2890625" style="91" customWidth="1"/>
-    <col min="7" max="8" width="20.859375" style="91" customWidth="1"/>
-    <col min="9" max="9" width="12.859375" style="91"/>
-    <col min="10" max="10" width="12" style="91"/>
-    <col min="11" max="16384" width="18.0390625" style="91"/>
+    <col min="1" max="1" width="17.4296875" style="92"/>
+    <col min="2" max="2" width="13.4296875" style="92" customWidth="1"/>
+    <col min="3" max="3" width="36" style="92" customWidth="1"/>
+    <col min="4" max="4" width="21.2890625" style="90" customWidth="1"/>
+    <col min="5" max="5" width="33.2890625" style="92" customWidth="1"/>
+    <col min="6" max="6" width="17.2890625" style="92" customWidth="1"/>
+    <col min="7" max="8" width="20.859375" style="92" customWidth="1"/>
+    <col min="9" max="9" width="12.859375" style="92"/>
+    <col min="10" max="10" width="12" style="92"/>
+    <col min="11" max="16384" width="18.0390625" style="92"/>
   </cols>
   <sheetData>
-    <row r="1" s="88" customFormat="1" ht="16" customHeight="1" spans="1:8">
-      <c r="A1" s="126" t="s">
+    <row r="1" s="89" customFormat="1" ht="16" customHeight="1" spans="1:8">
+      <c r="A1" s="123" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="127" t="s">
+      <c r="B1" s="124" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="127" t="s">
+      <c r="C1" s="124" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="127" t="s">
+      <c r="D1" s="124" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="127" t="s">
+      <c r="E1" s="124" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="127" t="s">
+      <c r="F1" s="124" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="127" t="s">
+      <c r="G1" s="124" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="127" t="s">
+      <c r="H1" s="124" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" s="88" customFormat="1" ht="120" customHeight="1" spans="1:8">
-      <c r="A2" s="128">
+    <row r="2" s="89" customFormat="1" ht="120" customHeight="1" spans="1:8">
+      <c r="A2" s="96">
         <v>45994</v>
       </c>
-      <c r="B2" s="96">
+      <c r="B2" s="103">
         <v>2518</v>
       </c>
-      <c r="C2" s="129" t="s">
+      <c r="C2" s="125" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="130">
+      <c r="D2" s="126">
         <v>4</v>
       </c>
-      <c r="E2" s="113" t="str">
+      <c r="E2" s="112" t="str">
         <f>_xlfn.DISPIMG("ID_AF642E9448564DC2B9A94250BEBF50D7",1)</f>
         <v>=DISPIMG("ID_AF642E9448564DC2B9A94250BEBF50D7",1)</v>
       </c>
-      <c r="F2" s="114">
+      <c r="F2" s="117">
         <v>178000</v>
       </c>
-      <c r="G2" s="139">
+      <c r="G2" s="133">
         <f t="shared" ref="G2:G8" si="0">SUM(D2*F2)</f>
         <v>712000</v>
       </c>
-      <c r="H2" s="139">
+      <c r="H2" s="133">
         <f>SUM(G2:G3)</f>
         <v>1897000</v>
       </c>
     </row>
-    <row r="3" s="88" customFormat="1" ht="120" customHeight="1" spans="1:8">
-      <c r="A3" s="131"/>
-      <c r="B3" s="96"/>
-      <c r="C3" s="129" t="s">
+    <row r="3" s="89" customFormat="1" ht="120" customHeight="1" spans="1:8">
+      <c r="A3" s="100"/>
+      <c r="B3" s="103"/>
+      <c r="C3" s="125" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="130">
+      <c r="D3" s="126">
         <v>3</v>
       </c>
-      <c r="E3" s="140"/>
-      <c r="F3" s="114">
+      <c r="E3" s="115"/>
+      <c r="F3" s="117">
         <v>395000</v>
       </c>
-      <c r="G3" s="139">
+      <c r="G3" s="133">
         <f t="shared" si="0"/>
         <v>1185000</v>
       </c>
-      <c r="H3" s="141"/>
-    </row>
-    <row r="4" s="88" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A4" s="128"/>
-      <c r="B4" s="132"/>
-      <c r="C4" s="133"/>
-      <c r="D4" s="130"/>
-      <c r="E4" s="113"/>
-      <c r="F4" s="139"/>
-      <c r="G4" s="139">
+      <c r="H3" s="134"/>
+    </row>
+    <row r="4" s="89" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A4" s="96"/>
+      <c r="B4" s="97"/>
+      <c r="C4" s="127"/>
+      <c r="D4" s="126"/>
+      <c r="E4" s="112"/>
+      <c r="F4" s="133"/>
+      <c r="G4" s="133">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H4" s="139">
+      <c r="H4" s="133">
         <f>SUM(G4:G7)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" s="88" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A5" s="131"/>
-      <c r="B5" s="134"/>
-      <c r="C5" s="96"/>
-      <c r="D5" s="96"/>
-      <c r="E5" s="140"/>
-      <c r="F5" s="142"/>
-      <c r="G5" s="139">
+    <row r="5" s="89" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A5" s="100"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="103"/>
+      <c r="D5" s="103"/>
+      <c r="E5" s="115"/>
+      <c r="F5" s="135"/>
+      <c r="G5" s="133">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H5" s="141"/>
-    </row>
-    <row r="6" s="88" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A6" s="131"/>
-      <c r="B6" s="134"/>
-      <c r="C6" s="96"/>
-      <c r="D6" s="96"/>
-      <c r="E6" s="140"/>
-      <c r="F6" s="142"/>
-      <c r="G6" s="139">
+      <c r="H5" s="134"/>
+    </row>
+    <row r="6" s="89" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A6" s="100"/>
+      <c r="B6" s="101"/>
+      <c r="C6" s="103"/>
+      <c r="D6" s="103"/>
+      <c r="E6" s="115"/>
+      <c r="F6" s="135"/>
+      <c r="G6" s="133">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="141"/>
-    </row>
-    <row r="7" s="88" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A7" s="131"/>
-      <c r="B7" s="134"/>
-      <c r="C7" s="132"/>
-      <c r="D7" s="132"/>
-      <c r="E7" s="140"/>
-      <c r="F7" s="142"/>
-      <c r="G7" s="139">
+      <c r="H6" s="134"/>
+    </row>
+    <row r="7" s="89" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A7" s="100"/>
+      <c r="B7" s="101"/>
+      <c r="C7" s="97"/>
+      <c r="D7" s="97"/>
+      <c r="E7" s="115"/>
+      <c r="F7" s="135"/>
+      <c r="G7" s="133">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H7" s="141"/>
-    </row>
-    <row r="8" s="88" customFormat="1" ht="258" customHeight="1" spans="1:8">
-      <c r="A8" s="95"/>
-      <c r="B8" s="96"/>
-      <c r="C8" s="96"/>
-      <c r="D8" s="96"/>
-      <c r="E8" s="143"/>
-      <c r="F8" s="144"/>
-      <c r="G8" s="114">
+      <c r="H7" s="134"/>
+    </row>
+    <row r="8" s="89" customFormat="1" ht="258" customHeight="1" spans="1:8">
+      <c r="A8" s="128"/>
+      <c r="B8" s="103"/>
+      <c r="C8" s="103"/>
+      <c r="D8" s="103"/>
+      <c r="E8" s="136"/>
+      <c r="F8" s="137"/>
+      <c r="G8" s="117">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="114">
+      <c r="H8" s="117">
         <f>SUM(G8)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9" s="88" customFormat="1" ht="18" customHeight="1" spans="1:8">
-      <c r="A9" s="135" t="s">
+    <row r="9" s="89" customFormat="1" ht="18" customHeight="1" spans="1:8">
+      <c r="A9" s="129" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="136"/>
-      <c r="C9" s="137"/>
-      <c r="D9" s="138"/>
-      <c r="E9" s="145"/>
-      <c r="F9" s="145"/>
-      <c r="G9" s="146"/>
-      <c r="H9" s="147">
+      <c r="B9" s="130"/>
+      <c r="C9" s="131"/>
+      <c r="D9" s="132"/>
+      <c r="E9" s="138"/>
+      <c r="F9" s="138"/>
+      <c r="G9" s="139"/>
+      <c r="H9" s="140">
         <f>SUM(H2:H8)</f>
         <v>1897000</v>
       </c>
@@ -2350,413 +2275,398 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="20.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="19.859375" style="89"/>
-    <col min="2" max="2" width="18.859375" style="89" customWidth="1"/>
-    <col min="3" max="3" width="43.0390625" style="90" customWidth="1"/>
-    <col min="4" max="4" width="14.4296875" style="89" customWidth="1"/>
-    <col min="5" max="5" width="58.9609375" style="91" customWidth="1"/>
-    <col min="6" max="6" width="19.5234375" style="91" customWidth="1"/>
-    <col min="7" max="8" width="20.859375" style="91" customWidth="1"/>
-    <col min="9" max="9" width="12.859375" style="91"/>
-    <col min="10" max="16384" width="9.140625" style="91"/>
+    <col min="1" max="1" width="19.859375" style="90"/>
+    <col min="2" max="2" width="18.859375" style="90" customWidth="1"/>
+    <col min="3" max="3" width="43.0390625" style="91" customWidth="1"/>
+    <col min="4" max="4" width="14.4296875" style="90" customWidth="1"/>
+    <col min="5" max="5" width="58.9609375" style="92" customWidth="1"/>
+    <col min="6" max="6" width="19.5234375" style="92" customWidth="1"/>
+    <col min="7" max="8" width="20.859375" style="92" customWidth="1"/>
+    <col min="9" max="9" width="12.859375" style="92"/>
+    <col min="10" max="16384" width="9.140625" style="92"/>
   </cols>
   <sheetData>
-    <row r="1" s="88" customFormat="1" ht="16" customHeight="1" spans="1:8">
-      <c r="A1" s="92" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="93" t="s">
+    <row r="1" s="89" customFormat="1" ht="16" customHeight="1" spans="1:8">
+      <c r="A1" s="93" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="94" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="94" t="s">
+      <c r="C1" s="95" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="93" t="s">
+      <c r="D1" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="93" t="s">
+      <c r="E1" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="93" t="s">
+      <c r="F1" s="94" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="93" t="s">
+      <c r="G1" s="94" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="93" t="s">
+      <c r="H1" s="94" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" s="88" customFormat="1" ht="227.8" customHeight="1" spans="1:8">
-      <c r="A2" s="95">
-        <v>45975</v>
-      </c>
-      <c r="B2" s="96">
-        <v>221</v>
-      </c>
-      <c r="C2" s="97" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="98">
-        <v>3</v>
-      </c>
-      <c r="E2" s="113"/>
-      <c r="F2" s="114">
+    <row r="2" s="89" customFormat="1" ht="32" customHeight="1" spans="1:8">
+      <c r="A2" s="96">
+        <v>46002</v>
+      </c>
+      <c r="B2" s="141" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="98" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="99">
+        <v>1</v>
+      </c>
+      <c r="E2" s="112" t="str">
+        <f>_xlfn.DISPIMG("ID_515301B36E6F4ABA90C3BE145E0FA8EF",1)</f>
+        <v>=DISPIMG("ID_515301B36E6F4ABA90C3BE145E0FA8EF",1)</v>
+      </c>
+      <c r="F2" s="113">
+        <v>295000</v>
+      </c>
+      <c r="G2" s="113">
+        <f t="shared" ref="G2:G16" si="0">D2*F2</f>
+        <v>295000</v>
+      </c>
+      <c r="H2" s="114">
+        <f>SUM(G2:G10)</f>
+        <v>5630000</v>
+      </c>
+    </row>
+    <row r="3" s="89" customFormat="1" ht="32" customHeight="1" spans="1:8">
+      <c r="A3" s="100"/>
+      <c r="B3" s="101"/>
+      <c r="C3" s="98" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="99">
+        <v>4</v>
+      </c>
+      <c r="E3" s="115"/>
+      <c r="F3" s="113">
+        <v>150000</v>
+      </c>
+      <c r="G3" s="113">
+        <f t="shared" si="0"/>
+        <v>600000</v>
+      </c>
+      <c r="H3" s="116"/>
+    </row>
+    <row r="4" s="89" customFormat="1" ht="32" customHeight="1" spans="1:8">
+      <c r="A4" s="100"/>
+      <c r="B4" s="101"/>
+      <c r="C4" s="98" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="99">
+        <v>4</v>
+      </c>
+      <c r="E4" s="115"/>
+      <c r="F4" s="113">
+        <v>460000</v>
+      </c>
+      <c r="G4" s="113">
+        <f t="shared" si="0"/>
+        <v>1840000</v>
+      </c>
+      <c r="H4" s="116"/>
+    </row>
+    <row r="5" s="89" customFormat="1" ht="32" customHeight="1" spans="1:8">
+      <c r="A5" s="100"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="98" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="99">
+        <v>2</v>
+      </c>
+      <c r="E5" s="115"/>
+      <c r="F5" s="113">
+        <v>340000</v>
+      </c>
+      <c r="G5" s="113">
+        <f t="shared" si="0"/>
+        <v>680000</v>
+      </c>
+      <c r="H5" s="116"/>
+    </row>
+    <row r="6" s="89" customFormat="1" ht="32" customHeight="1" spans="1:8">
+      <c r="A6" s="100"/>
+      <c r="B6" s="101"/>
+      <c r="C6" s="98" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="99">
+        <v>1</v>
+      </c>
+      <c r="E6" s="115"/>
+      <c r="F6" s="117">
+        <v>340000</v>
+      </c>
+      <c r="G6" s="113">
+        <f t="shared" si="0"/>
+        <v>340000</v>
+      </c>
+      <c r="H6" s="116"/>
+    </row>
+    <row r="7" s="89" customFormat="1" ht="32" customHeight="1" spans="1:8">
+      <c r="A7" s="100"/>
+      <c r="B7" s="101"/>
+      <c r="C7" s="102" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="103">
+        <v>5</v>
+      </c>
+      <c r="E7" s="115"/>
+      <c r="F7" s="117">
         <v>55000</v>
       </c>
-      <c r="G2" s="115">
-        <f t="shared" ref="G2:G12" si="0">D2*F2</f>
-        <v>165000</v>
-      </c>
-      <c r="H2" s="116">
-        <f>SUM(G2:G2)</f>
-        <v>165000</v>
-      </c>
-    </row>
-    <row r="3" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
-      <c r="A3" s="99">
-        <v>46002</v>
-      </c>
-      <c r="B3" s="148" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="101" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="98">
+      <c r="G7" s="113">
+        <f t="shared" si="0"/>
+        <v>275000</v>
+      </c>
+      <c r="H7" s="116"/>
+    </row>
+    <row r="8" s="89" customFormat="1" ht="32" customHeight="1" spans="1:8">
+      <c r="A8" s="100"/>
+      <c r="B8" s="101"/>
+      <c r="C8" s="102" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="103">
+        <v>500</v>
+      </c>
+      <c r="E8" s="115"/>
+      <c r="F8" s="117">
+        <v>1000</v>
+      </c>
+      <c r="G8" s="113">
+        <f t="shared" si="0"/>
+        <v>500000</v>
+      </c>
+      <c r="H8" s="116"/>
+    </row>
+    <row r="9" s="89" customFormat="1" ht="32" customHeight="1" spans="1:8">
+      <c r="A9" s="100"/>
+      <c r="B9" s="101"/>
+      <c r="C9" s="102" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="103">
+        <v>500</v>
+      </c>
+      <c r="E9" s="115"/>
+      <c r="F9" s="117">
+        <v>1500</v>
+      </c>
+      <c r="G9" s="113">
+        <f t="shared" si="0"/>
+        <v>750000</v>
+      </c>
+      <c r="H9" s="116"/>
+    </row>
+    <row r="10" s="89" customFormat="1" ht="32" customHeight="1" spans="1:8">
+      <c r="A10" s="104"/>
+      <c r="B10" s="105"/>
+      <c r="C10" s="106" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="107">
+        <v>10</v>
+      </c>
+      <c r="E10" s="118"/>
+      <c r="F10" s="117">
+        <v>35000</v>
+      </c>
+      <c r="G10" s="113">
+        <f t="shared" si="0"/>
+        <v>350000</v>
+      </c>
+      <c r="H10" s="116"/>
+    </row>
+    <row r="11" s="89" customFormat="1" ht="70" customHeight="1" spans="1:8">
+      <c r="A11" s="108">
+        <v>46003</v>
+      </c>
+      <c r="B11" s="109">
+        <v>938</v>
+      </c>
+      <c r="C11" s="106" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="107">
+        <v>4</v>
+      </c>
+      <c r="E11" s="109" t="str">
+        <f>_xlfn.DISPIMG("ID_6BB72733B67442EAB4426B445D61C75A",1)</f>
+        <v>=DISPIMG("ID_6BB72733B67442EAB4426B445D61C75A",1)</v>
+      </c>
+      <c r="F11" s="117">
+        <v>500000</v>
+      </c>
+      <c r="G11" s="113">
+        <f t="shared" si="0"/>
+        <v>2000000</v>
+      </c>
+      <c r="H11" s="119">
+        <f>SUM(G11:G14)</f>
+        <v>2740000</v>
+      </c>
+    </row>
+    <row r="12" s="89" customFormat="1" ht="70" customHeight="1" spans="1:8">
+      <c r="A12" s="108"/>
+      <c r="B12" s="109"/>
+      <c r="C12" s="106" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" s="107">
         <v>1</v>
       </c>
-      <c r="E3" s="117"/>
-      <c r="F3" s="115">
-        <v>295000</v>
-      </c>
-      <c r="G3" s="115">
-        <f t="shared" si="0"/>
-        <v>295000</v>
-      </c>
-      <c r="H3" s="118">
-        <f>SUM(G3:G11)</f>
-        <v>5630000</v>
-      </c>
-    </row>
-    <row r="4" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
-      <c r="A4" s="102"/>
-      <c r="B4" s="103"/>
-      <c r="C4" s="101" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="98">
-        <v>4</v>
-      </c>
-      <c r="E4" s="119"/>
-      <c r="F4" s="115">
-        <v>150000</v>
-      </c>
-      <c r="G4" s="115">
-        <f t="shared" si="0"/>
-        <v>600000</v>
-      </c>
-      <c r="H4" s="120"/>
-    </row>
-    <row r="5" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
-      <c r="A5" s="102"/>
-      <c r="B5" s="103"/>
-      <c r="C5" s="101" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="98">
-        <v>4</v>
-      </c>
-      <c r="E5" s="119"/>
-      <c r="F5" s="115">
-        <v>460000</v>
-      </c>
-      <c r="G5" s="115">
-        <f t="shared" si="0"/>
-        <v>1840000</v>
-      </c>
-      <c r="H5" s="120"/>
-    </row>
-    <row r="6" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
-      <c r="A6" s="102"/>
-      <c r="B6" s="103"/>
-      <c r="C6" s="101" t="s">
+      <c r="E12" s="109"/>
+      <c r="F12" s="117">
+        <v>340000</v>
+      </c>
+      <c r="G12" s="113">
+        <f t="shared" si="0"/>
+        <v>340000</v>
+      </c>
+      <c r="H12" s="119"/>
+    </row>
+    <row r="13" s="89" customFormat="1" ht="70" customHeight="1" spans="1:8">
+      <c r="A13" s="108"/>
+      <c r="B13" s="109"/>
+      <c r="C13" s="106" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="98">
+      <c r="D13" s="107">
         <v>2</v>
       </c>
-      <c r="E6" s="119"/>
-      <c r="F6" s="115">
-        <v>340000</v>
-      </c>
-      <c r="G6" s="115">
-        <f t="shared" si="0"/>
-        <v>680000</v>
-      </c>
-      <c r="H6" s="120"/>
-    </row>
-    <row r="7" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
-      <c r="A7" s="102"/>
-      <c r="B7" s="103"/>
-      <c r="C7" s="101" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="98">
-        <v>1</v>
-      </c>
-      <c r="E7" s="119"/>
-      <c r="F7" s="114">
-        <v>340000</v>
-      </c>
-      <c r="G7" s="115">
-        <f t="shared" si="0"/>
-        <v>340000</v>
-      </c>
-      <c r="H7" s="120"/>
-    </row>
-    <row r="8" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
-      <c r="A8" s="102"/>
-      <c r="B8" s="103"/>
-      <c r="C8" s="104" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="96">
-        <v>5</v>
-      </c>
-      <c r="E8" s="119"/>
-      <c r="F8" s="114">
-        <v>55000</v>
-      </c>
-      <c r="G8" s="115">
-        <f t="shared" si="0"/>
-        <v>275000</v>
-      </c>
-      <c r="H8" s="120"/>
-    </row>
-    <row r="9" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
-      <c r="A9" s="102"/>
-      <c r="B9" s="103"/>
-      <c r="C9" s="104" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="96">
-        <v>500</v>
-      </c>
-      <c r="E9" s="119"/>
-      <c r="F9" s="114">
-        <v>1000</v>
-      </c>
-      <c r="G9" s="115">
+      <c r="E13" s="109"/>
+      <c r="F13" s="117">
+        <v>25000</v>
+      </c>
+      <c r="G13" s="113">
+        <f t="shared" si="0"/>
+        <v>50000</v>
+      </c>
+      <c r="H13" s="119"/>
+    </row>
+    <row r="14" s="89" customFormat="1" ht="70" customHeight="1" spans="1:8">
+      <c r="A14" s="108"/>
+      <c r="B14" s="109"/>
+      <c r="C14" s="106" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" s="107">
+        <v>10</v>
+      </c>
+      <c r="E14" s="109"/>
+      <c r="F14" s="117">
+        <v>35000</v>
+      </c>
+      <c r="G14" s="113">
+        <f t="shared" si="0"/>
+        <v>350000</v>
+      </c>
+      <c r="H14" s="120"/>
+    </row>
+    <row r="15" s="89" customFormat="1" ht="353.9" customHeight="1" spans="1:8">
+      <c r="A15" s="110">
+        <v>46008</v>
+      </c>
+      <c r="B15" s="142" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="106" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="107">
+        <v>20</v>
+      </c>
+      <c r="E15" s="111" t="str">
+        <f>_xlfn.DISPIMG("ID_360A81D236BB40E99ADBAD1BA0483D4A",1)</f>
+        <v>=DISPIMG("ID_360A81D236BB40E99ADBAD1BA0483D4A",1)</v>
+      </c>
+      <c r="F15" s="107">
+        <v>25000</v>
+      </c>
+      <c r="G15" s="113">
         <f t="shared" si="0"/>
         <v>500000</v>
       </c>
-      <c r="H9" s="120"/>
-    </row>
-    <row r="10" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
-      <c r="A10" s="102"/>
-      <c r="B10" s="103"/>
-      <c r="C10" s="104" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" s="96">
-        <v>500</v>
-      </c>
-      <c r="E10" s="119"/>
-      <c r="F10" s="114">
-        <v>1500</v>
-      </c>
-      <c r="G10" s="115">
-        <f t="shared" si="0"/>
-        <v>750000</v>
-      </c>
-      <c r="H10" s="120"/>
-    </row>
-    <row r="11" s="88" customFormat="1" ht="32" customHeight="1" spans="1:8">
-      <c r="A11" s="105"/>
-      <c r="B11" s="106"/>
-      <c r="C11" s="107" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="108">
+      <c r="H15" s="121">
+        <f>SUM(G15)</f>
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="16" s="89" customFormat="1" ht="308.9" customHeight="1" spans="1:8">
+      <c r="A16" s="110">
+        <v>46013</v>
+      </c>
+      <c r="B16" s="142" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="106" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="107">
         <v>10</v>
       </c>
-      <c r="E11" s="121"/>
-      <c r="F11" s="114">
+      <c r="E16" s="111" t="str">
+        <f>_xlfn.DISPIMG("ID_8F95A6AC7B8A4D948EAF5FC4A9DACCAC",1)</f>
+        <v>=DISPIMG("ID_8F95A6AC7B8A4D948EAF5FC4A9DACCAC",1)</v>
+      </c>
+      <c r="F16" s="107">
         <v>35000</v>
       </c>
-      <c r="G11" s="115">
-        <f>D11*F11</f>
+      <c r="G16" s="113">
+        <f t="shared" si="0"/>
         <v>350000</v>
       </c>
-      <c r="H11" s="120"/>
-    </row>
-    <row r="12" s="88" customFormat="1" ht="70" customHeight="1" spans="1:8">
-      <c r="A12" s="109">
-        <v>46003</v>
-      </c>
-      <c r="B12" s="110">
-        <v>938</v>
-      </c>
-      <c r="C12" s="107" t="s">
-        <v>22</v>
-      </c>
-      <c r="D12" s="108">
-        <v>4</v>
-      </c>
-      <c r="E12" s="110"/>
-      <c r="F12" s="114">
-        <v>500000</v>
-      </c>
-      <c r="G12" s="115">
-        <f>D12*F12</f>
-        <v>2000000</v>
-      </c>
-      <c r="H12" s="122">
-        <f>SUM(G12:G15)</f>
-        <v>2740000</v>
-      </c>
-    </row>
-    <row r="13" s="88" customFormat="1" ht="70" customHeight="1" spans="1:8">
-      <c r="A13" s="109"/>
-      <c r="B13" s="110"/>
-      <c r="C13" s="107" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="108">
-        <v>1</v>
-      </c>
-      <c r="E13" s="110"/>
-      <c r="F13" s="114">
-        <v>340000</v>
-      </c>
-      <c r="G13" s="115">
-        <f>D13*F13</f>
-        <v>340000</v>
-      </c>
-      <c r="H13" s="122"/>
-    </row>
-    <row r="14" s="88" customFormat="1" ht="70" customHeight="1" spans="1:8">
-      <c r="A14" s="109"/>
-      <c r="B14" s="110"/>
-      <c r="C14" s="107" t="s">
-        <v>16</v>
-      </c>
-      <c r="D14" s="108">
-        <v>2</v>
-      </c>
-      <c r="E14" s="110"/>
-      <c r="F14" s="114">
-        <v>25000</v>
-      </c>
-      <c r="G14" s="115">
-        <f>D14*F14</f>
-        <v>50000</v>
-      </c>
-      <c r="H14" s="122"/>
-    </row>
-    <row r="15" s="88" customFormat="1" ht="70" customHeight="1" spans="1:8">
-      <c r="A15" s="109"/>
-      <c r="B15" s="110"/>
-      <c r="C15" s="107" t="s">
-        <v>21</v>
-      </c>
-      <c r="D15" s="108">
-        <v>10</v>
-      </c>
-      <c r="E15" s="110"/>
-      <c r="F15" s="114">
-        <v>35000</v>
-      </c>
-      <c r="G15" s="115">
-        <f>D15*F15</f>
+      <c r="H16" s="121">
+        <f>SUM(G16)</f>
         <v>350000</v>
       </c>
-      <c r="H15" s="123"/>
-    </row>
-    <row r="16" s="88" customFormat="1" ht="353.9" customHeight="1" spans="1:8">
-      <c r="A16" s="111">
-        <v>46008</v>
-      </c>
-      <c r="B16" s="149" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="107" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" s="108">
-        <v>20</v>
-      </c>
-      <c r="E16" s="112"/>
-      <c r="F16" s="108">
-        <v>25000</v>
-      </c>
-      <c r="G16" s="115">
-        <f>D16*F16</f>
-        <v>500000</v>
-      </c>
-      <c r="H16" s="124">
-        <f>SUM(G16)</f>
-        <v>500000</v>
-      </c>
-    </row>
-    <row r="17" s="88" customFormat="1" ht="308.9" customHeight="1" spans="1:8">
-      <c r="A17" s="111">
-        <v>46013</v>
-      </c>
-      <c r="B17" s="149" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="107" t="s">
-        <v>26</v>
-      </c>
-      <c r="D17" s="108">
-        <v>10</v>
-      </c>
-      <c r="E17" s="112"/>
-      <c r="F17" s="108">
-        <v>35000</v>
-      </c>
-      <c r="G17" s="115">
-        <f>D17*F17</f>
-        <v>350000</v>
-      </c>
-      <c r="H17" s="124">
-        <f>SUM(G17)</f>
-        <v>350000</v>
-      </c>
-    </row>
-    <row r="18" s="88" customFormat="1" spans="1:8">
-      <c r="A18" s="108"/>
-      <c r="B18" s="108"/>
-      <c r="C18" s="107"/>
-      <c r="D18" s="108"/>
-      <c r="E18" s="108"/>
-      <c r="F18" s="108"/>
-      <c r="G18" s="115"/>
-      <c r="H18" s="125">
-        <f>SUM(H2:H17)</f>
-        <v>9385000</v>
+    </row>
+    <row r="17" s="89" customFormat="1" spans="1:8">
+      <c r="A17" s="107"/>
+      <c r="B17" s="107"/>
+      <c r="C17" s="106"/>
+      <c r="D17" s="107"/>
+      <c r="E17" s="107"/>
+      <c r="F17" s="107"/>
+      <c r="G17" s="113"/>
+      <c r="H17" s="122">
+        <f>SUM(H2:H16)</f>
+        <v>9220000</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A3:A11"/>
-    <mergeCell ref="A12:A15"/>
-    <mergeCell ref="B3:B11"/>
-    <mergeCell ref="B12:B15"/>
-    <mergeCell ref="E3:E11"/>
-    <mergeCell ref="E12:E15"/>
-    <mergeCell ref="H3:H11"/>
-    <mergeCell ref="H12:H15"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A2:A10"/>
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="B2:B10"/>
+    <mergeCell ref="B11:B14"/>
+    <mergeCell ref="E2:E10"/>
+    <mergeCell ref="E11:E14"/>
+    <mergeCell ref="H2:H10"/>
+    <mergeCell ref="H11:H14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2776,33 +2686,33 @@
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="52" t="s">
+      <c r="B1" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="52" t="s">
+      <c r="C1" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="52" t="s">
+      <c r="D1" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="52" t="s">
+      <c r="E1" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="52" t="s">
+      <c r="F1" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="52" t="s">
+      <c r="G1" s="53" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A2" s="53"/>
-      <c r="B2" s="40"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="55"/>
+      <c r="A2" s="54"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="56"/>
       <c r="E2" s="74"/>
       <c r="F2" s="75"/>
       <c r="G2" s="76">
@@ -2811,94 +2721,94 @@
       </c>
     </row>
     <row r="3" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A3" s="53"/>
-      <c r="B3" s="40"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="57"/>
+      <c r="A3" s="54"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="58"/>
       <c r="E3" s="74"/>
       <c r="F3" s="77"/>
       <c r="G3" s="76"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="53"/>
-      <c r="B4" s="58" t="s">
+      <c r="A4" s="54"/>
+      <c r="B4" s="59" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="58"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="59"/>
-      <c r="F4" s="59"/>
-      <c r="G4" s="59">
+      <c r="C4" s="59"/>
+      <c r="D4" s="60"/>
+      <c r="E4" s="60"/>
+      <c r="F4" s="60"/>
+      <c r="G4" s="60">
         <f>SUM(G2:G3)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="53"/>
-      <c r="B5" s="58" t="s">
+      <c r="A5" s="54"/>
+      <c r="B5" s="59" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="58"/>
-      <c r="D5" s="59"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="59"/>
-      <c r="G5" s="59">
+      <c r="C5" s="59"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60">
         <f>G4*11%</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="53"/>
-      <c r="B6" s="58" t="s">
+      <c r="A6" s="54"/>
+      <c r="B6" s="59" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="58"/>
-      <c r="D6" s="59"/>
-      <c r="E6" s="59"/>
-      <c r="F6" s="59"/>
+      <c r="C6" s="59"/>
+      <c r="D6" s="60"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="60"/>
       <c r="G6" s="78">
         <v>243</v>
       </c>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="53"/>
-      <c r="B7" s="58" t="s">
+      <c r="A7" s="54"/>
+      <c r="B7" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="58"/>
-      <c r="D7" s="59"/>
+      <c r="C7" s="59"/>
+      <c r="D7" s="60"/>
       <c r="E7" s="79"/>
       <c r="F7" s="79"/>
       <c r="G7" s="79"/>
     </row>
     <row r="8" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A8" s="53"/>
-      <c r="B8" s="60"/>
-      <c r="C8" s="61"/>
-      <c r="D8" s="62"/>
+      <c r="A8" s="54"/>
+      <c r="B8" s="61"/>
+      <c r="C8" s="62"/>
+      <c r="D8" s="49"/>
       <c r="E8" s="80"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="81"/>
+      <c r="F8" s="81"/>
+      <c r="G8" s="82"/>
     </row>
     <row r="9" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A9" s="53"/>
+      <c r="A9" s="54"/>
       <c r="B9" s="63"/>
-      <c r="C9" s="61"/>
-      <c r="D9" s="62"/>
-      <c r="E9" s="82"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="81"/>
+      <c r="C9" s="62"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="83"/>
+      <c r="F9" s="81"/>
+      <c r="G9" s="82"/>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="64"/>
-      <c r="B10" s="58" t="s">
+      <c r="B10" s="59" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="58"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="83"/>
-      <c r="F10" s="59"/>
-      <c r="G10" s="59">
+      <c r="C10" s="59"/>
+      <c r="D10" s="60"/>
+      <c r="E10" s="84"/>
+      <c r="F10" s="60"/>
+      <c r="G10" s="60">
         <f>SUM(G8:G9)</f>
         <v>0</v>
       </c>
@@ -2909,20 +2819,20 @@
         <v>28</v>
       </c>
       <c r="C11" s="67"/>
-      <c r="D11" s="59"/>
-      <c r="E11" s="83"/>
-      <c r="F11" s="59"/>
-      <c r="G11" s="59"/>
+      <c r="D11" s="60"/>
+      <c r="E11" s="84"/>
+      <c r="F11" s="60"/>
+      <c r="G11" s="60"/>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="64"/>
-      <c r="B12" s="58" t="s">
+      <c r="B12" s="59" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="58"/>
-      <c r="D12" s="59"/>
-      <c r="E12" s="83"/>
-      <c r="F12" s="59"/>
+      <c r="C12" s="59"/>
+      <c r="D12" s="60"/>
+      <c r="E12" s="84"/>
+      <c r="F12" s="60"/>
       <c r="G12" s="78"/>
     </row>
     <row r="13" spans="1:7">
@@ -2931,9 +2841,9 @@
         <v>7</v>
       </c>
       <c r="C13" s="70"/>
-      <c r="D13" s="59"/>
+      <c r="D13" s="60"/>
       <c r="E13" s="79"/>
-      <c r="F13" s="84"/>
+      <c r="F13" s="85"/>
       <c r="G13" s="79">
         <f>SUM(G10:G12)</f>
         <v>0</v>
@@ -2946,12 +2856,12 @@
       <c r="B14" s="72"/>
       <c r="C14" s="72"/>
       <c r="D14" s="73"/>
-      <c r="E14" s="85">
+      <c r="E14" s="86">
         <f>G7+G13</f>
         <v>0</v>
       </c>
-      <c r="F14" s="86"/>
-      <c r="G14" s="87"/>
+      <c r="F14" s="87"/>
+      <c r="G14" s="88"/>
     </row>
   </sheetData>
   <mergeCells count="20">
@@ -2984,262 +2894,489 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E32"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelCol="4"/>
+  <dimension ref="A1:D33"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="10.5703125" style="12" customWidth="1"/>
     <col min="2" max="2" width="12.6015625" style="37" customWidth="1"/>
-    <col min="3" max="3" width="36.125" style="12" customWidth="1"/>
-    <col min="4" max="4" width="18.828125" style="12" customWidth="1"/>
-    <col min="5" max="5" width="12.2890625" style="12" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="12"/>
+    <col min="3" max="3" width="18.828125" style="38" customWidth="1"/>
+    <col min="4" max="4" width="18.828125" style="39" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" s="36" customFormat="1" ht="19" customHeight="1" spans="1:5">
-      <c r="A1" s="38" t="s">
+    <row r="1" s="36" customFormat="1" ht="19" customHeight="1" spans="1:4">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="38" t="s">
+      <c r="C1" s="42" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="43" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" s="12" customFormat="1" spans="1:4">
+      <c r="A2" s="44">
+        <v>45992</v>
+      </c>
+      <c r="B2" s="143" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="46">
+        <f>D2/8000</f>
+        <v>8</v>
+      </c>
+      <c r="D2" s="47">
+        <v>64000</v>
+      </c>
+    </row>
+    <row r="3" s="12" customFormat="1" spans="1:4">
+      <c r="A3" s="44">
+        <v>45993</v>
+      </c>
+      <c r="B3" s="143" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="46">
+        <f t="shared" ref="C3:C30" si="0">D3/8000</f>
+        <v>6</v>
+      </c>
+      <c r="D3" s="48">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="4" s="12" customFormat="1" spans="1:4">
+      <c r="A4" s="44">
+        <v>45994</v>
+      </c>
+      <c r="B4" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="46">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D4" s="48"/>
+    </row>
+    <row r="5" s="12" customFormat="1" spans="1:4">
+      <c r="A5" s="44">
+        <v>45995</v>
+      </c>
+      <c r="B5" s="143" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="46">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="D1" s="38" t="s">
+      <c r="D5" s="48">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="6" s="12" customFormat="1" spans="1:4">
+      <c r="A6" s="44">
+        <v>45996</v>
+      </c>
+      <c r="B6" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="46">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D6" s="48"/>
+    </row>
+    <row r="7" s="12" customFormat="1" spans="1:4">
+      <c r="A7" s="44">
+        <v>45997</v>
+      </c>
+      <c r="B7" s="143" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="46">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="D7" s="48">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="8" s="12" customFormat="1" spans="1:4">
+      <c r="A8" s="44">
+        <v>45998</v>
+      </c>
+      <c r="B8" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="46">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D8" s="48"/>
+    </row>
+    <row r="9" s="12" customFormat="1" spans="1:4">
+      <c r="A9" s="44">
+        <v>45999</v>
+      </c>
+      <c r="B9" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="46">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D9" s="48"/>
+    </row>
+    <row r="10" s="12" customFormat="1" spans="1:4">
+      <c r="A10" s="44">
+        <v>46000</v>
+      </c>
+      <c r="B10" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="46">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D10" s="48"/>
+    </row>
+    <row r="11" s="12" customFormat="1" spans="1:4">
+      <c r="A11" s="44">
+        <v>46001</v>
+      </c>
+      <c r="B11" s="143" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="46">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="E1" s="38" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" s="12" customFormat="1" ht="263.65" customHeight="1" spans="1:5">
-      <c r="A2" s="40"/>
-      <c r="B2" s="41"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="42"/>
-    </row>
-    <row r="3" s="12" customFormat="1" ht="255.1" customHeight="1" spans="1:5">
-      <c r="A3" s="40"/>
-      <c r="B3" s="41"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="49"/>
-    </row>
-    <row r="4" s="12" customFormat="1" ht="249.95" customHeight="1" spans="1:5">
-      <c r="A4" s="40"/>
-      <c r="B4" s="41"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="49"/>
-    </row>
-    <row r="5" s="12" customFormat="1" ht="256.25" customHeight="1" spans="1:5">
-      <c r="A5" s="40"/>
-      <c r="B5" s="41"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="49"/>
-    </row>
-    <row r="6" s="12" customFormat="1" ht="253.85" customHeight="1" spans="1:5">
-      <c r="A6" s="40"/>
-      <c r="B6" s="41"/>
-      <c r="C6" s="42"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="49"/>
-    </row>
-    <row r="7" s="12" customFormat="1" ht="254.65" customHeight="1" spans="1:5">
-      <c r="A7" s="40"/>
-      <c r="B7" s="41"/>
-      <c r="C7" s="42"/>
-      <c r="D7" s="44"/>
-      <c r="E7" s="49"/>
-    </row>
-    <row r="8" s="12" customFormat="1" ht="255.35" customHeight="1" spans="1:5">
-      <c r="A8" s="40"/>
-      <c r="B8" s="41"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="49"/>
-    </row>
-    <row r="9" s="12" customFormat="1" ht="266.95" customHeight="1" spans="1:5">
-      <c r="A9" s="40"/>
-      <c r="B9" s="41"/>
-      <c r="C9" s="42"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="49"/>
-    </row>
-    <row r="10" s="12" customFormat="1" ht="261.95" customHeight="1" spans="1:5">
-      <c r="A10" s="40"/>
-      <c r="B10" s="41"/>
-      <c r="C10" s="42"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="49"/>
-    </row>
-    <row r="11" s="12" customFormat="1" ht="261.9" customHeight="1" spans="1:5">
-      <c r="A11" s="40"/>
-      <c r="B11" s="41"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="49"/>
-    </row>
-    <row r="12" s="12" customFormat="1" ht="270.7" customHeight="1" spans="1:5">
-      <c r="A12" s="40"/>
-      <c r="B12" s="41"/>
-      <c r="C12" s="42"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="49"/>
-    </row>
-    <row r="13" s="12" customFormat="1" ht="261.1" customHeight="1" spans="1:5">
-      <c r="A13" s="40"/>
-      <c r="B13" s="41"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="49"/>
-    </row>
-    <row r="14" s="12" customFormat="1" ht="257.15" customHeight="1" spans="1:5">
-      <c r="A14" s="40"/>
-      <c r="B14" s="41"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="49"/>
-    </row>
-    <row r="15" s="12" customFormat="1" ht="263.55" customHeight="1" spans="1:5">
-      <c r="A15" s="40"/>
-      <c r="B15" s="41"/>
-      <c r="C15" s="42"/>
-      <c r="D15" s="44"/>
-      <c r="E15" s="49"/>
-    </row>
-    <row r="16" s="12" customFormat="1" ht="270.35" customHeight="1" spans="1:5">
-      <c r="A16" s="40"/>
-      <c r="B16" s="41"/>
-      <c r="C16" s="42"/>
-      <c r="D16" s="44"/>
-      <c r="E16" s="49"/>
-    </row>
-    <row r="17" s="12" customFormat="1" ht="261.7" customHeight="1" spans="1:5">
-      <c r="A17" s="40"/>
-      <c r="B17" s="41"/>
-      <c r="C17" s="42"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="49"/>
-    </row>
-    <row r="18" s="12" customFormat="1" ht="260" customHeight="1" spans="1:5">
-      <c r="A18" s="40"/>
-      <c r="B18" s="41"/>
-      <c r="C18" s="42"/>
-      <c r="D18" s="44"/>
-      <c r="E18" s="49"/>
-    </row>
-    <row r="19" s="12" customFormat="1" ht="263.2" customHeight="1" spans="1:5">
-      <c r="A19" s="40"/>
-      <c r="B19" s="41"/>
-      <c r="C19" s="42"/>
-      <c r="D19" s="44"/>
-      <c r="E19" s="49"/>
-    </row>
-    <row r="20" s="12" customFormat="1" ht="289.95" customHeight="1" spans="1:5">
-      <c r="A20" s="40"/>
-      <c r="B20" s="41"/>
-      <c r="C20" s="42"/>
-      <c r="D20" s="44"/>
-      <c r="E20" s="49"/>
-    </row>
-    <row r="21" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A21" s="40"/>
-      <c r="B21" s="41"/>
-      <c r="C21" s="42"/>
-      <c r="D21" s="44"/>
-      <c r="E21" s="49"/>
-    </row>
-    <row r="22" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A22" s="40"/>
-      <c r="B22" s="41"/>
-      <c r="C22" s="42"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="49"/>
-    </row>
-    <row r="23" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A23" s="40"/>
-      <c r="B23" s="41"/>
-      <c r="C23" s="42"/>
-      <c r="D23" s="44"/>
-      <c r="E23" s="49"/>
-    </row>
-    <row r="24" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A24" s="40"/>
-      <c r="B24" s="41"/>
-      <c r="C24" s="42"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="42"/>
-    </row>
-    <row r="25" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A25" s="40"/>
-      <c r="B25" s="41"/>
-      <c r="C25" s="42"/>
-      <c r="D25" s="43"/>
-      <c r="E25" s="42"/>
-    </row>
-    <row r="26" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A26" s="40"/>
-      <c r="B26" s="41"/>
-      <c r="C26" s="42"/>
-      <c r="D26" s="43"/>
-      <c r="E26" s="42"/>
-    </row>
-    <row r="27" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A27" s="40">
-        <v>45960</v>
-      </c>
-      <c r="B27" s="41"/>
-      <c r="C27" s="42"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="42"/>
-    </row>
-    <row r="28" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A28" s="40">
-        <v>45961</v>
-      </c>
-      <c r="B28" s="41"/>
-      <c r="C28" s="42"/>
-      <c r="D28" s="43"/>
-      <c r="E28" s="42"/>
-    </row>
-    <row r="29" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A29" s="40"/>
-      <c r="B29" s="41"/>
-      <c r="C29" s="42"/>
-      <c r="D29" s="43"/>
-      <c r="E29" s="42"/>
-    </row>
-    <row r="30" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A30" s="40"/>
-      <c r="B30" s="41"/>
-      <c r="C30" s="42"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="42"/>
-    </row>
-    <row r="31" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A31" s="40"/>
-      <c r="B31" s="41"/>
-      <c r="C31" s="42"/>
-      <c r="D31" s="43"/>
-      <c r="E31" s="42"/>
-    </row>
-    <row r="32" s="12" customFormat="1" spans="1:5">
-      <c r="A32" s="45"/>
-      <c r="B32" s="46"/>
-      <c r="C32" s="47">
-        <f>SUM(D2:D31)</f>
+      <c r="D11" s="48">
+        <v>56000</v>
+      </c>
+    </row>
+    <row r="12" s="12" customFormat="1" spans="1:4">
+      <c r="A12" s="44">
+        <v>46002</v>
+      </c>
+      <c r="B12" s="143" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="46">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="D12" s="48">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="13" s="12" customFormat="1" spans="1:4">
+      <c r="A13" s="44">
+        <v>46003</v>
+      </c>
+      <c r="B13" s="143" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="46">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="D13" s="48">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="14" s="12" customFormat="1" spans="1:4">
+      <c r="A14" s="44">
+        <v>46004</v>
+      </c>
+      <c r="B14" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="46">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D32" s="48"/>
-      <c r="E32" s="50"/>
+      <c r="D14" s="48"/>
+    </row>
+    <row r="15" s="12" customFormat="1" spans="1:4">
+      <c r="A15" s="44">
+        <v>46005</v>
+      </c>
+      <c r="B15" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="46">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D15" s="48"/>
+    </row>
+    <row r="16" s="12" customFormat="1" spans="1:4">
+      <c r="A16" s="44">
+        <v>46006</v>
+      </c>
+      <c r="B16" s="143" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="46">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="D16" s="48">
+        <v>96000</v>
+      </c>
+    </row>
+    <row r="17" s="12" customFormat="1" spans="1:4">
+      <c r="A17" s="44">
+        <v>46007</v>
+      </c>
+      <c r="B17" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="46">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D17" s="48"/>
+    </row>
+    <row r="18" s="12" customFormat="1" spans="1:4">
+      <c r="A18" s="44">
+        <v>46008</v>
+      </c>
+      <c r="B18" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="46">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D18" s="48"/>
+    </row>
+    <row r="19" s="12" customFormat="1" spans="1:4">
+      <c r="A19" s="44">
+        <v>46009</v>
+      </c>
+      <c r="B19" s="143" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="46">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="D19" s="48">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="20" s="12" customFormat="1" spans="1:4">
+      <c r="A20" s="44">
+        <v>46010</v>
+      </c>
+      <c r="B20" s="143" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" s="46">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="D20" s="48">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="21" s="12" customFormat="1" spans="1:4">
+      <c r="A21" s="44">
+        <v>46011</v>
+      </c>
+      <c r="B21" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="46">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D21" s="48"/>
+    </row>
+    <row r="22" s="12" customFormat="1" spans="1:4">
+      <c r="A22" s="44">
+        <v>46012</v>
+      </c>
+      <c r="B22" s="45">
+        <v>1452</v>
+      </c>
+      <c r="C22" s="46">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="D22" s="48">
+        <v>64000</v>
+      </c>
+    </row>
+    <row r="23" s="12" customFormat="1" spans="1:4">
+      <c r="A23" s="44">
+        <v>46013</v>
+      </c>
+      <c r="B23" s="143" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" s="46">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="D23" s="48">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="24" s="12" customFormat="1" spans="1:4">
+      <c r="A24" s="44">
+        <v>46014</v>
+      </c>
+      <c r="B24" s="45">
+        <v>1453</v>
+      </c>
+      <c r="C24" s="46">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="D24" s="47">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="25" s="12" customFormat="1" spans="1:4">
+      <c r="A25" s="44">
+        <v>46015</v>
+      </c>
+      <c r="B25" s="45">
+        <v>1454</v>
+      </c>
+      <c r="C25" s="46">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="D25" s="47">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="26" s="12" customFormat="1" spans="1:4">
+      <c r="A26" s="44">
+        <v>46016</v>
+      </c>
+      <c r="B26" s="45">
+        <v>1455</v>
+      </c>
+      <c r="C26" s="46">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="D26" s="47">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="27" s="12" customFormat="1" spans="1:4">
+      <c r="A27" s="44">
+        <v>46017</v>
+      </c>
+      <c r="B27" s="45">
+        <v>1456</v>
+      </c>
+      <c r="C27" s="46">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="D27" s="47">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="28" s="12" customFormat="1" spans="1:4">
+      <c r="A28" s="44">
+        <v>46018</v>
+      </c>
+      <c r="B28" s="45">
+        <v>1457</v>
+      </c>
+      <c r="C28" s="46">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="D28" s="47">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="29" s="12" customFormat="1" spans="1:4">
+      <c r="A29" s="44">
+        <v>46019</v>
+      </c>
+      <c r="B29" s="45">
+        <v>1458</v>
+      </c>
+      <c r="C29" s="46">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="D29" s="47">
+        <v>56000</v>
+      </c>
+    </row>
+    <row r="30" s="12" customFormat="1" spans="1:4">
+      <c r="A30" s="44">
+        <v>46020</v>
+      </c>
+      <c r="B30" s="45">
+        <v>1459</v>
+      </c>
+      <c r="C30" s="46">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="D30" s="47">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="31" s="12" customFormat="1" spans="1:4">
+      <c r="A31" s="44">
+        <v>46021</v>
+      </c>
+      <c r="B31" s="45">
+        <v>1460</v>
+      </c>
+      <c r="C31" s="46">
+        <f>D31/8000</f>
+        <v>6</v>
+      </c>
+      <c r="D31" s="47">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="32" s="12" customFormat="1" spans="1:4">
+      <c r="A32" s="44">
+        <v>46022</v>
+      </c>
+      <c r="B32" s="49">
+        <v>1461</v>
+      </c>
+      <c r="C32" s="46">
+        <f>D32/8000</f>
+        <v>1</v>
+      </c>
+      <c r="D32" s="47">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="50" t="s">
+        <v>10</v>
+      </c>
+      <c r="B33" s="50"/>
+      <c r="C33" s="50"/>
+      <c r="D33" s="51">
+        <f>SUM(D2:D32)</f>
+        <v>944000</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="C32:E32"/>
+  <mergeCells count="1">
+    <mergeCell ref="A33:C33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -3265,10 +3402,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="D1" s="15" t="s">
         <v>4</v>
@@ -3288,7 +3425,7 @@
         <v>45992</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="C2" s="18">
         <v>1</v>
@@ -3309,7 +3446,7 @@
     <row r="3" s="12" customFormat="1" ht="80" customHeight="1" spans="1:7">
       <c r="A3" s="20"/>
       <c r="B3" s="21" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="C3" s="22">
         <v>1</v>
@@ -3329,7 +3466,7 @@
         <v>46003</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="C4" s="22">
         <v>3</v>
@@ -3350,7 +3487,7 @@
     <row r="5" s="12" customFormat="1" ht="48" customHeight="1" spans="1:7">
       <c r="A5" s="26"/>
       <c r="B5" s="21" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="C5" s="22">
         <v>1</v>
@@ -3368,7 +3505,7 @@
     <row r="6" s="12" customFormat="1" ht="48" customHeight="1" spans="1:7">
       <c r="A6" s="26"/>
       <c r="B6" s="21" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="C6" s="22">
         <v>1</v>
@@ -3386,7 +3523,7 @@
     <row r="7" s="12" customFormat="1" ht="48" customHeight="1" spans="1:7">
       <c r="A7" s="26"/>
       <c r="B7" s="21" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="C7" s="22">
         <v>3</v>
@@ -3404,7 +3541,7 @@
     <row r="8" s="12" customFormat="1" ht="48" customHeight="1" spans="1:7">
       <c r="A8" s="27"/>
       <c r="B8" s="21" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="C8" s="22">
         <v>1</v>
@@ -3424,7 +3561,7 @@
         <v>46013</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="C9" s="22">
         <v>3</v>
@@ -3452,8 +3589,8 @@
       <c r="E10" s="29"/>
       <c r="F10" s="30"/>
       <c r="G10" s="35">
-        <f>SUM(G2:G8)</f>
-        <v>850000</v>
+        <f>SUM(G2:G9)</f>
+        <v>1300000</v>
       </c>
     </row>
   </sheetData>
@@ -3484,13 +3621,13 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:3">
       <c r="A1" s="3" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -3498,7 +3635,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="C2" s="8">
         <f>'Anugrah (Bag, Cup, Box)'!H9</f>
@@ -3510,11 +3647,11 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="C3" s="8">
-        <f>'UD Abdi Jaya (Bag, Cup, Box)'!H18</f>
-        <v>9385000</v>
+        <f>'UD Abdi Jaya (Bag, Cup, Box)'!H17</f>
+        <v>9220000</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -3522,7 +3659,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C4" s="8">
         <f>'PT. SUPARMA JAYA TBK (Tissue)'!E14</f>
@@ -3534,11 +3671,11 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" s="9">
-        <f>'Vickel Laundry'!C32</f>
-        <v>0</v>
+        <v>59</v>
+      </c>
+      <c r="C5" s="9" t="e">
+        <f>'Vickel Laundry'!#REF!</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -3546,11 +3683,11 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C6" s="9">
         <f>'Dishy Soap'!G10</f>
-        <v>850000</v>
+        <v>1300000</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -3558,9 +3695,9 @@
         <v>7</v>
       </c>
       <c r="B7" s="7"/>
-      <c r="C7" s="10">
+      <c r="C7" s="10" t="e">
         <f>SUM(C2:C5)</f>
-        <v>11282000</v>
+        <v>#REF!</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
10 jan 2026 09.14
</commit_message>
<xml_diff>
--- a/DECEMBER/DECEMBER FLOOR.xlsx
+++ b/DECEMBER/DECEMBER FLOOR.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="16060" activeTab="3"/>
+    <workbookView windowHeight="17020"/>
   </bookViews>
   <sheets>
     <sheet name="Anugrah (Bag, Cup, Box)" sheetId="1" r:id="rId1"/>
@@ -36,39 +36,13 @@
   <etc:cellImage>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="ID_AF642E9448564DC2B9A94250BEBF50D7" descr="WhatsApp Image 2025-12-03 at 18.16.51_a036882e"/>
+        <xdr:cNvPr id="9" name="ID_6BB72733B67442EAB4426B445D61C75A"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip r:embed="rId1"/>
-        <a:srcRect l="1437" t="10012" b="11665"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5927090" y="226060"/>
-          <a:ext cx="2122170" cy="3007360"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-  </etc:cellImage>
-  <etc:cellImage>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="ID_6BB72733B67442EAB4426B445D61C75A"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
         <a:srcRect t="25750" r="2659" b="15363"/>
         <a:stretch>
           <a:fillRect/>
@@ -98,7 +72,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
+        <a:blip r:embed="rId2"/>
         <a:srcRect t="19236" b="11470"/>
         <a:stretch>
           <a:fillRect/>
@@ -124,7 +98,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId4"/>
+        <a:blip r:embed="rId3"/>
         <a:srcRect l="2346" t="14598" b="17958"/>
         <a:stretch>
           <a:fillRect/>
@@ -150,7 +124,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId5"/>
+        <a:blip r:embed="rId4"/>
         <a:srcRect t="26542" b="15720"/>
         <a:stretch>
           <a:fillRect/>
@@ -1704,6 +1678,50 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>297815</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>27305</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>2418080</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>1508760</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="ID_AF642E9448564DC2B9A94250BEBF50D7" descr="WhatsApp Image 2025-12-03 at 18.16.51_a036882e"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:srcRect l="1437" t="10012" b="11665"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7462520" y="230505"/>
+          <a:ext cx="2120265" cy="3005455"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>43180</xdr:colOff>
       <xdr:row>8</xdr:row>
@@ -2134,10 +2152,7 @@
       <c r="D2" s="126">
         <v>4</v>
       </c>
-      <c r="E2" s="112" t="str">
-        <f>_xlfn.DISPIMG("ID_AF642E9448564DC2B9A94250BEBF50D7",1)</f>
-        <v>=DISPIMG("ID_AF642E9448564DC2B9A94250BEBF50D7",1)</v>
-      </c>
+      <c r="E2" s="112"/>
       <c r="F2" s="117">
         <v>178000</v>
       </c>
@@ -2269,6 +2284,7 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2941,7 +2957,7 @@
         <v>32</v>
       </c>
       <c r="C3" s="46">
-        <f t="shared" ref="C3:C30" si="0">D3/8000</f>
+        <f t="shared" ref="C3:C32" si="0">D3/8000</f>
         <v>6</v>
       </c>
       <c r="D3" s="48">
@@ -3138,9 +3154,11 @@
       </c>
       <c r="C17" s="46">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D17" s="48"/>
+        <v>5</v>
+      </c>
+      <c r="D17" s="48">
+        <v>40000</v>
+      </c>
     </row>
     <row r="18" s="12" customFormat="1" spans="1:4">
       <c r="A18" s="44">
@@ -3341,7 +3359,7 @@
         <v>1460</v>
       </c>
       <c r="C31" s="46">
-        <f>D31/8000</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="D31" s="47">
@@ -3356,7 +3374,7 @@
         <v>1461</v>
       </c>
       <c r="C32" s="46">
-        <f>D32/8000</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="D32" s="47">
@@ -3371,7 +3389,7 @@
       <c r="C33" s="50"/>
       <c r="D33" s="51">
         <f>SUM(D2:D32)</f>
-        <v>944000</v>
+        <v>984000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>